<commit_message>
Complete cleanup + final experimental setup
</commit_message>
<xml_diff>
--- a/figures/holding_period_scan_tp5_sl5.xlsx
+++ b/figures/holding_period_scan_tp5_sl5.xlsx
@@ -473,22 +473,22 @@
         <v>125</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4815591029926565</v>
+        <v>0.4803630847389745</v>
       </c>
       <c r="D2" t="n">
-        <v>0.06557786960755929</v>
+        <v>0.05580960270804816</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4528630273997842</v>
+        <v>0.4638273125529773</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.02869607559287235</v>
+        <v>0.01653577218599728</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8892984192475462</v>
+        <v>0.8695964152627146</v>
       </c>
     </row>
     <row r="3">
@@ -499,22 +499,22 @@
         <v>124</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4812004842997394</v>
+        <v>0.4799817854135178</v>
       </c>
       <c r="D3" t="n">
-        <v>0.06634774826941806</v>
+        <v>0.05651185182543623</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4524517674308425</v>
+        <v>0.463506362761046</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>0.02874871686889691</v>
+        <v>0.01647542265247176</v>
       </c>
       <c r="H3" t="n">
-        <v>0.8908033067099431</v>
+        <v>0.8710921690580786</v>
       </c>
     </row>
     <row r="4">
@@ -525,22 +525,22 @@
         <v>123</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4808747664043376</v>
+        <v>0.4796279176942089</v>
       </c>
       <c r="D4" t="n">
-        <v>0.06702221461848235</v>
+        <v>0.0572195872640539</v>
       </c>
       <c r="E4" t="n">
-        <v>0.45210301897718</v>
+        <v>0.4631524950417372</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0287717474271576</v>
+        <v>0.01647542265247176</v>
       </c>
       <c r="H4" t="n">
-        <v>0.8921145316893436</v>
+        <v>0.8725891870708968</v>
       </c>
     </row>
     <row r="5">
@@ -551,22 +551,22 @@
         <v>122</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4805293080304266</v>
+        <v>0.4792795362961297</v>
       </c>
       <c r="D5" t="n">
-        <v>0.06773945200431658</v>
+        <v>0.057894404775294</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4517312399652568</v>
+        <v>0.4628260589285763</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0.02879806806516988</v>
+        <v>0.01645347736755337</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8935008685736439</v>
+        <v>0.8740083106448806</v>
       </c>
     </row>
     <row r="6">
@@ -577,22 +577,22 @@
         <v>121</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4801838496565157</v>
+        <v>0.4789119527737469</v>
       </c>
       <c r="D6" t="n">
-        <v>0.06846326954965389</v>
+        <v>0.05863505814128923</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4513528807938305</v>
+        <v>0.4624529890849639</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0.02883096886268521</v>
+        <v>0.01645896368878297</v>
       </c>
       <c r="H6" t="n">
-        <v>0.894891466976665</v>
+        <v>0.8755557611417806</v>
       </c>
     </row>
     <row r="7">
@@ -603,22 +603,22 @@
         <v>120</v>
       </c>
       <c r="C7" t="n">
-        <v>0.479821940883847</v>
+        <v>0.4785087081633717</v>
       </c>
       <c r="D7" t="n">
-        <v>0.06927262916853104</v>
+        <v>0.05937845466789926</v>
       </c>
       <c r="E7" t="n">
-        <v>0.4509054299476219</v>
+        <v>0.4621128371687291</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>0.02891651093622505</v>
+        <v>0.01639587099464257</v>
       </c>
       <c r="H7" t="n">
-        <v>0.8964351660867496</v>
+        <v>0.877100147200546</v>
       </c>
     </row>
     <row r="8">
@@ -629,22 +629,22 @@
         <v>119</v>
       </c>
       <c r="C8" t="n">
-        <v>0.4794468717921723</v>
+        <v>0.4781219225166853</v>
       </c>
       <c r="D8" t="n">
-        <v>0.07009843918616587</v>
+        <v>0.06014379647942766</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4504546890216619</v>
+        <v>0.4617342810038871</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0.02899218277051041</v>
+        <v>0.0163876415127982</v>
       </c>
       <c r="H8" t="n">
-        <v>0.8980001183032066</v>
+        <v>0.8786787976294317</v>
       </c>
     </row>
     <row r="9">
@@ -655,22 +655,22 @@
         <v>118</v>
       </c>
       <c r="C9" t="n">
-        <v>0.4790685126207459</v>
+        <v>0.4776610715333994</v>
       </c>
       <c r="D9" t="n">
-        <v>0.07089134840628537</v>
+        <v>0.06095851518202242</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4500401389729687</v>
+        <v>0.4613804132845782</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>0.02902837364777722</v>
+        <v>0.01628065824882113</v>
       </c>
       <c r="H9" t="n">
-        <v>0.8994940050975084</v>
+        <v>0.8803496205677421</v>
       </c>
     </row>
     <row r="10">
@@ -681,22 +681,22 @@
         <v>117</v>
       </c>
       <c r="C10" t="n">
-        <v>0.4786704129708104</v>
+        <v>0.4772303953168762</v>
       </c>
       <c r="D10" t="n">
-        <v>0.07169412786565946</v>
+        <v>0.06178146336646157</v>
       </c>
       <c r="E10" t="n">
-        <v>0.4496354591635301</v>
+        <v>0.4609881413166622</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0.02903495380728027</v>
+        <v>0.01624225400021401</v>
       </c>
       <c r="H10" t="n">
-        <v>0.9009977009516951</v>
+        <v>0.8820243359120739</v>
       </c>
     </row>
     <row r="11">
@@ -707,22 +707,22 @@
         <v>116</v>
       </c>
       <c r="C11" t="n">
-        <v>0.4782920537993841</v>
+        <v>0.4767914896185086</v>
       </c>
       <c r="D11" t="n">
-        <v>0.07251664780354276</v>
+        <v>0.06267024740565585</v>
       </c>
       <c r="E11" t="n">
-        <v>0.4491912983970732</v>
+        <v>0.4605382629758355</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>0.02910075540231094</v>
+        <v>0.01625322664267315</v>
       </c>
       <c r="H11" t="n">
-        <v>0.9025264774078687</v>
+        <v>0.8838190004514528</v>
       </c>
     </row>
     <row r="12">
@@ -733,22 +733,22 @@
         <v>115</v>
       </c>
       <c r="C12" t="n">
-        <v>0.4778676335114363</v>
+        <v>0.4763498407595263</v>
       </c>
       <c r="D12" t="n">
-        <v>0.07342141973521438</v>
+        <v>0.06353708615993175</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4487109467533493</v>
+        <v>0.4601130730805419</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0.02915668675808697</v>
+        <v>0.01623676767898435</v>
       </c>
       <c r="H12" t="n">
-        <v>0.9041970248126471</v>
+        <v>0.8855568676679775</v>
       </c>
     </row>
     <row r="13">
@@ -759,22 +759,22 @@
         <v>114</v>
       </c>
       <c r="C13" t="n">
-        <v>0.4774563735424946</v>
+        <v>0.4759465961491511</v>
       </c>
       <c r="D13" t="n">
-        <v>0.07429000078961914</v>
+        <v>0.06440118175359286</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4482536256678862</v>
+        <v>0.459652222097256</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0.02920274787460847</v>
+        <v>0.0162943740518951</v>
       </c>
       <c r="H13" t="n">
-        <v>0.9057896613893144</v>
+        <v>0.8872753797340196</v>
       </c>
     </row>
     <row r="14">
@@ -785,22 +785,22 @@
         <v>113</v>
       </c>
       <c r="C14" t="n">
-        <v>0.4769793119785223</v>
+        <v>0.475543351538776</v>
       </c>
       <c r="D14" t="n">
-        <v>0.07521122312004842</v>
+        <v>0.06520767097434321</v>
       </c>
       <c r="E14" t="n">
-        <v>0.4478094649014292</v>
+        <v>0.4592489774868808</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>0.02916984707709314</v>
+        <v>0.01629437405189516</v>
       </c>
       <c r="H14" t="n">
-        <v>0.9074694128473682</v>
+        <v>0.8888690743711101</v>
       </c>
     </row>
     <row r="15">
@@ -811,22 +811,22 @@
         <v>112</v>
       </c>
       <c r="C15" t="n">
-        <v>0.4765351512120654</v>
+        <v>0.47508250055549</v>
       </c>
       <c r="D15" t="n">
-        <v>0.07605677361619245</v>
+        <v>0.06604433496185635</v>
       </c>
       <c r="E15" t="n">
-        <v>0.4474080751717421</v>
+        <v>0.4588731644826536</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>0.02912707604032322</v>
+        <v>0.01620933607283637</v>
       </c>
       <c r="H15" t="n">
-        <v>0.9090008387099227</v>
+        <v>0.8905126012727143</v>
       </c>
     </row>
     <row r="16">
@@ -837,22 +837,22 @@
         <v>111</v>
       </c>
       <c r="C16" t="n">
-        <v>0.4760778301266023</v>
+        <v>0.4746024474479005</v>
       </c>
       <c r="D16" t="n">
-        <v>0.07700102650488248</v>
+        <v>0.0669605506071986</v>
       </c>
       <c r="E16" t="n">
-        <v>0.4469211433685152</v>
+        <v>0.4584370019449009</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>0.02915668675808702</v>
+        <v>0.01616544550299964</v>
       </c>
       <c r="H16" t="n">
-        <v>0.9106965677920429</v>
+        <v>0.8922985261471452</v>
       </c>
     </row>
     <row r="17">
@@ -863,22 +863,22 @@
         <v>110</v>
       </c>
       <c r="C17" t="n">
-        <v>0.4756172189613876</v>
+        <v>0.4741141648584666</v>
       </c>
       <c r="D17" t="n">
-        <v>0.07786631747953571</v>
+        <v>0.06787950941315565</v>
       </c>
       <c r="E17" t="n">
-        <v>0.4465164635590766</v>
+        <v>0.4580063257283777</v>
       </c>
       <c r="F17" t="n">
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>0.029100755402311</v>
+        <v>0.0161078391300889</v>
       </c>
       <c r="H17" t="n">
-        <v>0.9122420972263878</v>
+        <v>0.8940765353057702</v>
       </c>
     </row>
     <row r="18">
@@ -889,22 +889,22 @@
         <v>109</v>
       </c>
       <c r="C18" t="n">
-        <v>0.475156607796173</v>
+        <v>0.4736203959478031</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0788072802884742</v>
+        <v>0.06884235878894945</v>
       </c>
       <c r="E18" t="n">
-        <v>0.4460361119153528</v>
+        <v>0.4575372452632474</v>
       </c>
       <c r="F18" t="n">
         <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>0.02912049588082016</v>
+        <v>0.01608315068455574</v>
       </c>
       <c r="H18" t="n">
-        <v>0.9139084099630734</v>
+        <v>0.8959245309190129</v>
       </c>
     </row>
     <row r="19">
@@ -915,22 +915,22 @@
         <v>108</v>
       </c>
       <c r="C19" t="n">
-        <v>0.4746795462322007</v>
+        <v>0.4730553048611549</v>
       </c>
       <c r="D19" t="n">
-        <v>0.07974495301766114</v>
+        <v>0.06992042091056473</v>
       </c>
       <c r="E19" t="n">
-        <v>0.4455755007501382</v>
+        <v>0.4570242742282803</v>
       </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>0.02910404548206247</v>
+        <v>0.01603103063287459</v>
       </c>
       <c r="H19" t="n">
-        <v>0.9155579044405764</v>
+        <v>0.8979769230186758</v>
       </c>
     </row>
     <row r="20">
@@ -941,22 +941,22 @@
         <v>107</v>
       </c>
       <c r="C20" t="n">
-        <v>0.4741597136314584</v>
+        <v>0.4725149022200399</v>
       </c>
       <c r="D20" t="n">
-        <v>0.08076816782038797</v>
+        <v>0.07095184930172846</v>
       </c>
       <c r="E20" t="n">
-        <v>0.4450721185481536</v>
+        <v>0.4565332484782316</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0.02908759508330483</v>
+        <v>0.01598165374180827</v>
       </c>
       <c r="H20" t="n">
-        <v>0.9173441652410601</v>
+        <v>0.8999237925166172</v>
       </c>
     </row>
     <row r="21">
@@ -967,22 +967,22 @@
         <v>106</v>
       </c>
       <c r="C21" t="n">
-        <v>0.4735905298344432</v>
+        <v>0.4719168932060141</v>
       </c>
       <c r="D21" t="n">
-        <v>0.08187363461690311</v>
+        <v>0.07209026095686928</v>
       </c>
       <c r="E21" t="n">
-        <v>0.4445358355486537</v>
+        <v>0.4559928458371166</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>0.02905469428578944</v>
+        <v>0.01592404736889746</v>
       </c>
       <c r="H21" t="n">
-        <v>0.9192586518182539</v>
+        <v>0.902053921270815</v>
       </c>
     </row>
     <row r="22">
@@ -993,22 +993,22 @@
         <v>105</v>
       </c>
       <c r="C22" t="n">
-        <v>0.4730443765956887</v>
+        <v>0.4713490589587511</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0829231700576422</v>
+        <v>0.07317380939971416</v>
       </c>
       <c r="E22" t="n">
-        <v>0.4440324533466691</v>
+        <v>0.4554771316415347</v>
       </c>
       <c r="F22" t="n">
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>0.02901192324901952</v>
+        <v>0.01587192731721637</v>
       </c>
       <c r="H22" t="n">
-        <v>0.9210615918960785</v>
+        <v>0.9040633446357331</v>
       </c>
     </row>
     <row r="23">
@@ -1019,22 +1019,22 @@
         <v>104</v>
       </c>
       <c r="C23" t="n">
-        <v>0.4725015134366857</v>
+        <v>0.4707976836751769</v>
       </c>
       <c r="D23" t="n">
-        <v>0.08395954517937515</v>
+        <v>0.07423541255764066</v>
       </c>
       <c r="E23" t="n">
-        <v>0.4435389413839391</v>
+        <v>0.4549669037671825</v>
       </c>
       <c r="F23" t="n">
         <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0289625720527466</v>
+        <v>0.01583077990799442</v>
       </c>
       <c r="H23" t="n">
-        <v>0.9228279350534279</v>
+        <v>0.9060151085476411</v>
       </c>
     </row>
     <row r="24">
@@ -1045,22 +1045,22 @@
         <v>103</v>
       </c>
       <c r="C24" t="n">
-        <v>0.4719454899586766</v>
+        <v>0.4701996746611511</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0850650119758903</v>
+        <v>0.07537931053401108</v>
       </c>
       <c r="E24" t="n">
-        <v>0.4429894980654331</v>
+        <v>0.4544210148048378</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>0.02895599189324349</v>
+        <v>0.01577865985631327</v>
       </c>
       <c r="H24" t="n">
-        <v>0.924695187639664</v>
+        <v>0.908099954884276</v>
       </c>
     </row>
     <row r="25">
@@ -1071,22 +1071,22 @@
         <v>102</v>
       </c>
       <c r="C25" t="n">
-        <v>0.4713335351248914</v>
+        <v>0.4696236109320437</v>
       </c>
       <c r="D25" t="n">
-        <v>0.08623299028768458</v>
+        <v>0.07656161275898865</v>
       </c>
       <c r="E25" t="n">
-        <v>0.442433474587424</v>
+        <v>0.4538147763089677</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0.02890006053746741</v>
+        <v>0.01580883462307603</v>
       </c>
       <c r="H25" t="n">
-        <v>0.9266525234077059</v>
+        <v>0.910233631961729</v>
       </c>
     </row>
     <row r="26">
@@ -1097,22 +1097,22 @@
         <v>101</v>
       </c>
       <c r="C26" t="n">
-        <v>0.4706919695733425</v>
+        <v>0.4689323344571148</v>
       </c>
       <c r="D26" t="n">
-        <v>0.08736806780196352</v>
+        <v>0.07779603503564737</v>
       </c>
       <c r="E26" t="n">
-        <v>0.441939962624694</v>
+        <v>0.4532716305072378</v>
       </c>
       <c r="F26" t="n">
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>0.02875200694864843</v>
+        <v>0.01566070394987695</v>
       </c>
       <c r="H26" t="n">
-        <v>0.9285410900219065</v>
+        <v>0.9124433399969795</v>
       </c>
     </row>
     <row r="27">
@@ -1123,22 +1123,22 @@
         <v>100</v>
       </c>
       <c r="C27" t="n">
-        <v>0.4700800147395573</v>
+        <v>0.4682849485520227</v>
       </c>
       <c r="D27" t="n">
-        <v>0.08856565683152159</v>
+        <v>0.0790139983486173</v>
       </c>
       <c r="E27" t="n">
-        <v>0.4413543284289211</v>
+        <v>0.45270105309936</v>
       </c>
       <c r="F27" t="n">
         <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>0.02872568631063616</v>
+        <v>0.01558389545266264</v>
       </c>
       <c r="H27" t="n">
-        <v>0.930512049327363</v>
+        <v>0.9146015784738277</v>
       </c>
     </row>
     <row r="28">
@@ -1149,22 +1149,22 @@
         <v>99</v>
       </c>
       <c r="C28" t="n">
-        <v>0.4694219987892507</v>
+        <v>0.4675717267921754</v>
       </c>
       <c r="D28" t="n">
-        <v>0.08984220777511646</v>
+        <v>0.08026487958896482</v>
       </c>
       <c r="E28" t="n">
-        <v>0.4407357934356329</v>
+        <v>0.4521633936188598</v>
       </c>
       <c r="F28" t="n">
         <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>0.02868620535361777</v>
+        <v>0.01540833317331564</v>
       </c>
       <c r="H28" t="n">
-        <v>0.9325937635016495</v>
+        <v>0.9167985520326524</v>
       </c>
     </row>
     <row r="29">
@@ -1175,22 +1175,22 @@
         <v>98</v>
       </c>
       <c r="C29" t="n">
-        <v>0.4686619903666465</v>
+        <v>0.4668310734261802</v>
       </c>
       <c r="D29" t="n">
-        <v>0.09122733135051193</v>
+        <v>0.0816254872539042</v>
       </c>
       <c r="E29" t="n">
-        <v>0.4401106782828416</v>
+        <v>0.4515434393199156</v>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0285513120838049</v>
+        <v>0.01528763410626455</v>
       </c>
       <c r="H29" t="n">
-        <v>0.9348328926068201</v>
+        <v>0.9191629890890132</v>
       </c>
     </row>
     <row r="30">
@@ -1201,22 +1201,22 @@
         <v>97</v>
       </c>
       <c r="C30" t="n">
-        <v>0.4678526307477693</v>
+        <v>0.4660547589721926</v>
       </c>
       <c r="D30" t="n">
-        <v>0.092721027557708</v>
+        <v>0.08303272864929515</v>
       </c>
       <c r="E30" t="n">
-        <v>0.4394263416945227</v>
+        <v>0.4509125123785123</v>
       </c>
       <c r="F30" t="n">
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>0.02842628905324668</v>
+        <v>0.0151422465936803</v>
       </c>
       <c r="H30" t="n">
-        <v>0.9372209590263577</v>
+        <v>0.9215828175278882</v>
       </c>
     </row>
     <row r="31">
@@ -1227,22 +1227,22 @@
         <v>96</v>
       </c>
       <c r="C31" t="n">
-        <v>0.4670761719264075</v>
+        <v>0.4652757013575902</v>
       </c>
       <c r="D31" t="n">
-        <v>0.09424762456241939</v>
+        <v>0.08449483325698202</v>
       </c>
       <c r="E31" t="n">
-        <v>0.4386762035111731</v>
+        <v>0.4502294653854278</v>
       </c>
       <c r="F31" t="n">
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0283999684152344</v>
+        <v>0.01504623597216237</v>
       </c>
       <c r="H31" t="n">
-        <v>0.9396310396744785</v>
+        <v>0.9240685197698018</v>
       </c>
     </row>
     <row r="32">
@@ -1253,22 +1253,22 @@
         <v>95</v>
       </c>
       <c r="C32" t="n">
-        <v>0.4663062932645488</v>
+        <v>0.4645323048309802</v>
       </c>
       <c r="D32" t="n">
-        <v>0.09572158029110625</v>
+        <v>0.08589658833114337</v>
       </c>
       <c r="E32" t="n">
-        <v>0.437972126444345</v>
+        <v>0.4495711068378765</v>
       </c>
       <c r="F32" t="n">
         <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>0.02833416682020373</v>
+        <v>0.01496119799310369</v>
       </c>
       <c r="H32" t="n">
-        <v>0.9419333705865908</v>
+        <v>0.9264255479521235</v>
       </c>
     </row>
     <row r="33">
@@ -1279,22 +1279,22 @@
         <v>94</v>
       </c>
       <c r="C33" t="n">
-        <v>0.4654640328481562</v>
+        <v>0.4637395314133038</v>
       </c>
       <c r="D33" t="n">
-        <v>0.09725804753507225</v>
+        <v>0.08744921723911857</v>
       </c>
       <c r="E33" t="n">
-        <v>0.4372779196167715</v>
+        <v>0.4488112513475777</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0281861132313847</v>
+        <v>0.01492828006572611</v>
       </c>
       <c r="H33" t="n">
-        <v>0.944309115757844</v>
+        <v>0.9290060667504286</v>
       </c>
     </row>
     <row r="34">
@@ -1305,22 +1305,22 @@
         <v>93</v>
       </c>
       <c r="C34" t="n">
-        <v>0.4645757113152423</v>
+        <v>0.4629056105864054</v>
       </c>
       <c r="D34" t="n">
-        <v>0.0989688890058695</v>
+        <v>0.08910059992922646</v>
       </c>
       <c r="E34" t="n">
-        <v>0.4364553996788882</v>
+        <v>0.4479937894843681</v>
       </c>
       <c r="F34" t="n">
         <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>0.02812031163635409</v>
+        <v>0.01491182110203737</v>
       </c>
       <c r="H34" t="n">
-        <v>0.9469197622466072</v>
+        <v>0.9317172722827494</v>
       </c>
     </row>
     <row r="35">
@@ -1331,22 +1331,22 @@
         <v>92</v>
       </c>
       <c r="C35" t="n">
-        <v>0.463703840181086</v>
+        <v>0.4620579739564331</v>
       </c>
       <c r="D35" t="n">
-        <v>0.1006599899981576</v>
+        <v>0.09076569842240834</v>
       </c>
       <c r="E35" t="n">
-        <v>0.4356361698207565</v>
+        <v>0.4471763276211586</v>
       </c>
       <c r="F35" t="n">
         <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>0.02806767036032953</v>
+        <v>0.01488164633527456</v>
       </c>
       <c r="H35" t="n">
-        <v>0.9494676380118192</v>
+        <v>0.9344171980011662</v>
       </c>
     </row>
     <row r="36">
@@ -1357,22 +1357,22 @@
         <v>91</v>
       </c>
       <c r="C36" t="n">
-        <v>0.4627760376911536</v>
+        <v>0.4611527309535501</v>
       </c>
       <c r="D36" t="n">
-        <v>0.1024826941805069</v>
+        <v>0.09246371484296777</v>
       </c>
       <c r="E36" t="n">
-        <v>0.4347412681283394</v>
+        <v>0.4463835542034822</v>
       </c>
       <c r="F36" t="n">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0280347695628142</v>
+        <v>0.01476917675006789</v>
       </c>
       <c r="H36" t="n">
-        <v>0.9521776857063621</v>
+        <v>0.9371372364164533</v>
       </c>
     </row>
     <row r="37">
@@ -1383,22 +1383,22 @@
         <v>90</v>
       </c>
       <c r="C37" t="n">
-        <v>0.4618449451214697</v>
+        <v>0.4602502311112818</v>
       </c>
       <c r="D37" t="n">
-        <v>0.104272497565341</v>
+        <v>0.09424951240320072</v>
       </c>
       <c r="E37" t="n">
-        <v>0.4338825573131893</v>
+        <v>0.4455002564855175</v>
       </c>
       <c r="F37" t="n">
         <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>0.02796238780828048</v>
+        <v>0.01474997462576427</v>
       </c>
       <c r="H37" t="n">
-        <v>0.9548049151181125</v>
+        <v>0.9399592125075619</v>
       </c>
     </row>
     <row r="38">
@@ -1409,22 +1409,22 @@
         <v>89</v>
       </c>
       <c r="C38" t="n">
-        <v>0.4608941120732766</v>
+        <v>0.4592901248961028</v>
       </c>
       <c r="D38" t="n">
-        <v>0.1060754612691812</v>
+        <v>0.09606822789081124</v>
       </c>
       <c r="E38" t="n">
-        <v>0.4330304266575422</v>
+        <v>0.444641647213086</v>
       </c>
       <c r="F38" t="n">
         <v>1</v>
       </c>
       <c r="G38" t="n">
-        <v>0.02786368541573447</v>
+        <v>0.0146484776830168</v>
       </c>
       <c r="H38" t="n">
-        <v>0.9574175893868442</v>
+        <v>0.94279614338955</v>
       </c>
     </row>
     <row r="39">
@@ -1435,22 +1435,22 @@
         <v>88</v>
       </c>
       <c r="C39" t="n">
-        <v>0.4598741873503014</v>
+        <v>0.4583327618415386</v>
       </c>
       <c r="D39" t="n">
-        <v>0.1079804174453189</v>
+        <v>0.09790614550272533</v>
       </c>
       <c r="E39" t="n">
-        <v>0.4321453952043798</v>
+        <v>0.4437610926557361</v>
       </c>
       <c r="F39" t="n">
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>0.02772879214592161</v>
+        <v>0.01457166918580249</v>
       </c>
       <c r="H39" t="n">
-        <v>0.9601417746848296</v>
+        <v>0.9456239097315409</v>
       </c>
     </row>
     <row r="40">
@@ -1461,22 +1461,22 @@
         <v>87</v>
       </c>
       <c r="C40" t="n">
-        <v>0.4589365146211144</v>
+        <v>0.4574467209629591</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1098656331429474</v>
+        <v>0.09974131995402463</v>
       </c>
       <c r="E40" t="n">
-        <v>0.4311978522359382</v>
+        <v>0.4428119590830163</v>
       </c>
       <c r="F40" t="n">
         <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>0.02773866238517619</v>
+        <v>0.01463476187994278</v>
       </c>
       <c r="H40" t="n">
-        <v>0.9627961713963686</v>
+        <v>0.9484070281893636</v>
       </c>
     </row>
     <row r="41">
@@ -1487,22 +1487,22 @@
         <v>86</v>
       </c>
       <c r="C41" t="n">
-        <v>0.4579593609349091</v>
+        <v>0.4564427241779433</v>
       </c>
       <c r="D41" t="n">
-        <v>0.1118002000368489</v>
+        <v>0.101738340881597</v>
       </c>
       <c r="E41" t="n">
-        <v>0.430240439028242</v>
+        <v>0.4418189349404597</v>
       </c>
       <c r="F41" t="n">
         <v>1</v>
       </c>
       <c r="G41" t="n">
-        <v>0.02771892190666703</v>
+        <v>0.01462378923748364</v>
       </c>
       <c r="H41" t="n">
-        <v>0.9654832045172768</v>
+        <v>0.9513942862675231</v>
       </c>
     </row>
     <row r="42">
@@ -1513,22 +1513,22 @@
         <v>85</v>
       </c>
       <c r="C42" t="n">
-        <v>0.4569690469296976</v>
+        <v>0.4553728915381725</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1136919958939805</v>
+        <v>0.1036777554362586</v>
       </c>
       <c r="E42" t="n">
-        <v>0.429338957176322</v>
+        <v>0.440949353025569</v>
       </c>
       <c r="F42" t="n">
         <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>0.02763008975337561</v>
+        <v>0.01442353851260347</v>
       </c>
       <c r="H42" t="n">
-        <v>0.9680765456331327</v>
+        <v>0.9542566656558367</v>
       </c>
     </row>
     <row r="43">
@@ -1539,22 +1539,22 @@
         <v>84</v>
       </c>
       <c r="C43" t="n">
-        <v>0.4559589924459769</v>
+        <v>0.4543634084319271</v>
       </c>
       <c r="D43" t="n">
-        <v>0.115682494143658</v>
+        <v>0.1056665468819865</v>
       </c>
       <c r="E43" t="n">
-        <v>0.4283585134103651</v>
+        <v>0.4399700446860864</v>
       </c>
       <c r="F43" t="n">
         <v>1</v>
       </c>
       <c r="G43" t="n">
-        <v>0.0276004790356118</v>
+        <v>0.01439336374584066</v>
       </c>
       <c r="H43" t="n">
-        <v>0.9707648623457301</v>
+        <v>0.9571470542349066</v>
       </c>
     </row>
     <row r="44">
@@ -1565,22 +1565,22 @@
         <v>83</v>
       </c>
       <c r="C44" t="n">
-        <v>0.45493577764325</v>
+        <v>0.453323750558919</v>
       </c>
       <c r="D44" t="n">
-        <v>0.1177453741478693</v>
+        <v>0.1077623215916915</v>
       </c>
       <c r="E44" t="n">
-        <v>0.4273188482088806</v>
+        <v>0.4389139278493895</v>
       </c>
       <c r="F44" t="n">
         <v>1</v>
       </c>
       <c r="G44" t="n">
-        <v>0.02761692943436944</v>
+        <v>0.01440982270952951</v>
       </c>
       <c r="H44" t="n">
-        <v>0.9735085973844346</v>
+        <v>0.9601468663977858</v>
       </c>
     </row>
     <row r="45">
@@ -1591,22 +1591,22 @@
         <v>82</v>
       </c>
       <c r="C45" t="n">
-        <v>0.4537579290922012</v>
+        <v>0.4521387051733266</v>
       </c>
       <c r="D45" t="n">
-        <v>0.1201109414892217</v>
+        <v>0.1100117132958252</v>
       </c>
       <c r="E45" t="n">
-        <v>0.4261311294185771</v>
+        <v>0.4378495815308482</v>
       </c>
       <c r="F45" t="n">
         <v>1</v>
       </c>
       <c r="G45" t="n">
-        <v>0.02762679967362408</v>
+        <v>0.01428912364247842</v>
       </c>
       <c r="H45" t="n">
-        <v>0.9766048082001979</v>
+        <v>0.9633179805749402</v>
       </c>
     </row>
     <row r="46">
@@ -1617,22 +1617,22 @@
         <v>81</v>
       </c>
       <c r="C46" t="n">
-        <v>0.4525833706209039</v>
+        <v>0.4508658786480607</v>
       </c>
       <c r="D46" t="n">
-        <v>0.1224896691495802</v>
+        <v>0.1124147219943875</v>
       </c>
       <c r="E46" t="n">
-        <v>0.424926960229516</v>
+        <v>0.4367193993575518</v>
       </c>
       <c r="F46" t="n">
         <v>1</v>
       </c>
       <c r="G46" t="n">
-        <v>0.02765641039138789</v>
+        <v>0.01414647929050894</v>
       </c>
       <c r="H46" t="n">
-        <v>0.9796642222304233</v>
+        <v>0.9666487952468232</v>
       </c>
     </row>
     <row r="47">
@@ -1643,22 +1643,22 @@
         <v>80</v>
       </c>
       <c r="C47" t="n">
-        <v>0.4513265601558182</v>
+        <v>0.4496424290138612</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1247960150554049</v>
+        <v>0.114653141056062</v>
       </c>
       <c r="E47" t="n">
-        <v>0.4238774247887769</v>
+        <v>0.4357044299300769</v>
       </c>
       <c r="F47" t="n">
         <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>0.0274491353670413</v>
+        <v>0.01393799908378435</v>
       </c>
       <c r="H47" t="n">
-        <v>0.9825876901760602</v>
+        <v>0.9697005659212987</v>
       </c>
     </row>
     <row r="48">
@@ -1669,22 +1669,22 @@
         <v>79</v>
       </c>
       <c r="C48" t="n">
-        <v>0.4500960703287448</v>
+        <v>0.4483174824369142</v>
       </c>
       <c r="D48" t="n">
-        <v>0.1271517121575027</v>
+        <v>0.1171329582518386</v>
       </c>
       <c r="E48" t="n">
-        <v>0.4227522175137525</v>
+        <v>0.4345495593112472</v>
       </c>
       <c r="F48" t="n">
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>0.02734385281499224</v>
+        <v>0.01376792312566694</v>
       </c>
       <c r="H48" t="n">
-        <v>0.9855200920161133</v>
+        <v>0.9730228607811582</v>
       </c>
     </row>
     <row r="49">
@@ -1695,22 +1695,22 @@
         <v>78</v>
       </c>
       <c r="C49" t="n">
-        <v>0.4488590003421683</v>
+        <v>0.4470089948236559</v>
       </c>
       <c r="D49" t="n">
-        <v>0.1296324322901587</v>
+        <v>0.1197115292297479</v>
       </c>
       <c r="E49" t="n">
-        <v>0.421508567367673</v>
+        <v>0.4332794759465962</v>
       </c>
       <c r="F49" t="n">
         <v>1</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0273504329744953</v>
+        <v>0.01372951887705975</v>
       </c>
       <c r="H49" t="n">
-        <v>0.9885503992792966</v>
+        <v>0.9764122363774246</v>
       </c>
     </row>
     <row r="50">
@@ -1721,22 +1721,22 @@
         <v>77</v>
       </c>
       <c r="C50" t="n">
-        <v>0.4473817545337299</v>
+        <v>0.4455990102676502</v>
       </c>
       <c r="D50" t="n">
-        <v>0.1323533282446767</v>
+        <v>0.1223285044562644</v>
       </c>
       <c r="E50" t="n">
-        <v>0.4202649172215934</v>
+        <v>0.4320724852760854</v>
       </c>
       <c r="F50" t="n">
         <v>1</v>
       </c>
       <c r="G50" t="n">
-        <v>0.02711683731213649</v>
+        <v>0.01352652499156481</v>
       </c>
       <c r="H50" t="n">
-        <v>0.9918189539709641</v>
+        <v>0.9797901249660503</v>
       </c>
     </row>
     <row r="51">
@@ -1747,22 +1747,22 @@
         <v>76</v>
       </c>
       <c r="C51" t="n">
-        <v>0.4460723027926197</v>
+        <v>0.4442521184057848</v>
       </c>
       <c r="D51" t="n">
-        <v>0.1349985523649093</v>
+        <v>0.1250058292163065</v>
       </c>
       <c r="E51" t="n">
-        <v>0.418929144842471</v>
+        <v>0.4307420523779088</v>
       </c>
       <c r="F51" t="n">
         <v>1</v>
       </c>
       <c r="G51" t="n">
-        <v>0.02714315795014871</v>
+        <v>0.01351006602787597</v>
       </c>
       <c r="H51" t="n">
-        <v>0.9949268462321721</v>
+        <v>0.9831769406585473</v>
       </c>
     </row>
     <row r="52">
@@ -1773,22 +1773,22 @@
         <v>75</v>
       </c>
       <c r="C52" t="n">
-        <v>0.4446411181007028</v>
+        <v>0.4427982432799423</v>
       </c>
       <c r="D52" t="n">
-        <v>0.1377029979206696</v>
+        <v>0.1277819077584812</v>
       </c>
       <c r="E52" t="n">
-        <v>0.4176558839786276</v>
+        <v>0.4294198489615765</v>
       </c>
       <c r="F52" t="n">
         <v>1</v>
       </c>
       <c r="G52" t="n">
-        <v>0.02698523412207515</v>
+        <v>0.01337839431836574</v>
       </c>
       <c r="H52" t="n">
-        <v>0.998048165728842</v>
+        <v>0.9866212510304491</v>
       </c>
     </row>
     <row r="53">
@@ -1799,22 +1799,22 @@
         <v>74</v>
       </c>
       <c r="C53" t="n">
-        <v>0.4431408417340036</v>
+        <v>0.4411742921959824</v>
       </c>
       <c r="D53" t="n">
-        <v>0.1405982681020188</v>
+        <v>0.130799384434758</v>
       </c>
       <c r="E53" t="n">
-        <v>0.4162608901639775</v>
+        <v>0.4280263233692596</v>
       </c>
       <c r="F53" t="n">
         <v>1</v>
       </c>
       <c r="G53" t="n">
-        <v>0.02687995157002609</v>
+        <v>0.01314796882672276</v>
       </c>
       <c r="H53" t="n">
-        <v>1.001319477323865</v>
+        <v>0.9902879908500148</v>
       </c>
     </row>
     <row r="54">
@@ -1825,22 +1825,22 @@
         <v>73</v>
       </c>
       <c r="C54" t="n">
-        <v>0.4415813439317769</v>
+        <v>0.4396326359304664</v>
       </c>
       <c r="D54" t="n">
-        <v>0.1435297291606349</v>
+        <v>0.1337427957744354</v>
       </c>
       <c r="E54" t="n">
-        <v>0.4148889269075882</v>
+        <v>0.4266245682950983</v>
       </c>
       <c r="F54" t="n">
         <v>1</v>
       </c>
       <c r="G54" t="n">
-        <v>0.02669241702418867</v>
+        <v>0.0130080676353681</v>
       </c>
       <c r="H54" t="n">
-        <v>1.004563526787678</v>
+        <v>0.9937862399760475</v>
       </c>
     </row>
     <row r="55">
@@ -1851,22 +1851,22 @@
         <v>72</v>
       </c>
       <c r="C55" t="n">
-        <v>0.4400119758902956</v>
+        <v>0.4380388596132692</v>
       </c>
       <c r="D55" t="n">
-        <v>0.1466355644460822</v>
+        <v>0.1367630156113271</v>
       </c>
       <c r="E55" t="n">
-        <v>0.4133524596636223</v>
+        <v>0.4251981247754038</v>
       </c>
       <c r="F55" t="n">
         <v>1</v>
       </c>
       <c r="G55" t="n">
-        <v>0.02665951622667329</v>
+        <v>0.01284073483786546</v>
       </c>
       <c r="H55" t="n">
-        <v>1.007919121559861</v>
+        <v>0.9972983938111872</v>
       </c>
     </row>
     <row r="56">
@@ -1877,22 +1877,22 @@
         <v>71</v>
       </c>
       <c r="C56" t="n">
-        <v>0.4383932566525413</v>
+        <v>0.4363490726745542</v>
       </c>
       <c r="D56" t="n">
-        <v>0.1497808806885479</v>
+        <v>0.1399615408881806</v>
       </c>
       <c r="E56" t="n">
-        <v>0.4118258626589109</v>
+        <v>0.4236893864372653</v>
       </c>
       <c r="F56" t="n">
         <v>1</v>
       </c>
       <c r="G56" t="n">
-        <v>0.02656739399363039</v>
+        <v>0.01265968623728891</v>
       </c>
       <c r="H56" t="n">
-        <v>1.011240644677013</v>
+        <v>1.000933716519817</v>
       </c>
     </row>
     <row r="57">
@@ -1903,22 +1903,22 @@
         <v>70</v>
       </c>
       <c r="C57" t="n">
-        <v>0.4367547969362777</v>
+        <v>0.4346510562539947</v>
       </c>
       <c r="D57" t="n">
-        <v>0.1530512199615719</v>
+        <v>0.1432588199471667</v>
       </c>
       <c r="E57" t="n">
-        <v>0.4101939831021504</v>
+        <v>0.4220901237988385</v>
       </c>
       <c r="F57" t="n">
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>0.02656081383412734</v>
+        <v>0.01256093245515622</v>
       </c>
       <c r="H57" t="n">
-        <v>1.014609035596669</v>
+        <v>1.004591016084537</v>
       </c>
     </row>
     <row r="58">
@@ -1929,22 +1929,22 @@
         <v>69</v>
       </c>
       <c r="C58" t="n">
-        <v>0.435047245545232</v>
+        <v>0.4328734881756062</v>
       </c>
       <c r="D58" t="n">
-        <v>0.1565255441791909</v>
+        <v>0.1466932570368928</v>
       </c>
       <c r="E58" t="n">
-        <v>0.4084272102755771</v>
+        <v>0.420433254787501</v>
       </c>
       <c r="F58" t="n">
         <v>1</v>
       </c>
       <c r="G58" t="n">
-        <v>0.0266200352696549</v>
+        <v>0.01244023338810513</v>
       </c>
       <c r="H58" t="n">
-        <v>1.018095067195067</v>
+        <v>1.008306539545091</v>
       </c>
     </row>
     <row r="59">
@@ -1955,22 +1955,22 @@
         <v>68</v>
       </c>
       <c r="C59" t="n">
-        <v>0.4332179612033796</v>
+        <v>0.4310931769366028</v>
       </c>
       <c r="D59" t="n">
-        <v>0.1600656699918406</v>
+        <v>0.1501304372872336</v>
       </c>
       <c r="E59" t="n">
-        <v>0.4067163688047798</v>
+        <v>0.4187763857761636</v>
       </c>
       <c r="F59" t="n">
         <v>1</v>
       </c>
       <c r="G59" t="n">
-        <v>0.02650159239859973</v>
+        <v>0.01231679116043921</v>
       </c>
       <c r="H59" t="n">
-        <v>1.021558710611006</v>
+        <v>1.011930711912869</v>
       </c>
     </row>
     <row r="60">
@@ -1981,22 +1981,22 @@
         <v>67</v>
       </c>
       <c r="C60" t="n">
-        <v>0.4313459058247572</v>
+        <v>0.4292826909308367</v>
       </c>
       <c r="D60" t="n">
-        <v>0.1637867501908246</v>
+        <v>0.1537431798169215</v>
       </c>
       <c r="E60" t="n">
-        <v>0.4048673439844182</v>
+        <v>0.4169741292522419</v>
       </c>
       <c r="F60" t="n">
         <v>1</v>
       </c>
       <c r="G60" t="n">
-        <v>0.02647856184033898</v>
+        <v>0.01230856167859484</v>
       </c>
       <c r="H60" t="n">
-        <v>1.025095728761331</v>
+        <v>1.015638446956844</v>
       </c>
     </row>
     <row r="61">
@@ -2007,22 +2007,22 @@
         <v>66</v>
       </c>
       <c r="C61" t="n">
-        <v>0.429246834943279</v>
+        <v>0.4272801836820347</v>
       </c>
       <c r="D61" t="n">
-        <v>0.1677611665306767</v>
+        <v>0.157509539341038</v>
       </c>
       <c r="E61" t="n">
-        <v>0.4029919985260443</v>
+        <v>0.4152102769769273</v>
       </c>
       <c r="F61" t="n">
         <v>1</v>
       </c>
       <c r="G61" t="n">
-        <v>0.02625483641723475</v>
+        <v>0.01206990670510749</v>
       </c>
       <c r="H61" t="n">
-        <v>1.028768228888003</v>
+        <v>1.01940037749027</v>
       </c>
     </row>
     <row r="62">
@@ -2033,22 +2033,22 @@
         <v>65</v>
       </c>
       <c r="C62" t="n">
-        <v>0.427259626773353</v>
+        <v>0.4253188238424548</v>
       </c>
       <c r="D62" t="n">
-        <v>0.1715941094412129</v>
+        <v>0.1612868715076136</v>
       </c>
       <c r="E62" t="n">
-        <v>0.4011462637854342</v>
+        <v>0.4133943046499315</v>
       </c>
       <c r="F62" t="n">
         <v>1</v>
       </c>
       <c r="G62" t="n">
-        <v>0.02611336298791883</v>
+        <v>0.01192451919252324</v>
       </c>
       <c r="H62" t="n">
-        <v>1.032200451724311</v>
+        <v>1.023064523536286</v>
       </c>
     </row>
     <row r="63">
@@ -2059,22 +2059,22 @@
         <v>64</v>
       </c>
       <c r="C63" t="n">
-        <v>0.4251539757323717</v>
+        <v>0.4232175628115202</v>
       </c>
       <c r="D63" t="n">
-        <v>0.1757165793698839</v>
+        <v>0.165352235538743</v>
       </c>
       <c r="E63" t="n">
-        <v>0.3991294448977443</v>
+        <v>0.4114302016497368</v>
       </c>
       <c r="F63" t="n">
         <v>1</v>
       </c>
       <c r="G63" t="n">
-        <v>0.02602453083462741</v>
+        <v>0.01178736116178336</v>
       </c>
       <c r="H63" t="n">
-        <v>1.035774619985765</v>
+        <v>1.026889985701657</v>
       </c>
     </row>
     <row r="64">
@@ -2085,22 +2085,22 @@
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>0.4228673703050562</v>
+        <v>0.4211217881018152</v>
       </c>
       <c r="D64" t="n">
-        <v>0.1800660648014108</v>
+        <v>0.1695026375489311</v>
       </c>
       <c r="E64" t="n">
-        <v>0.397066564893533</v>
+        <v>0.4093755743492537</v>
       </c>
       <c r="F64" t="n">
         <v>1</v>
       </c>
       <c r="G64" t="n">
-        <v>0.02580080541152313</v>
+        <v>0.01174621375256146</v>
       </c>
       <c r="H64" t="n">
-        <v>1.039422538537982</v>
+        <v>1.030670536972532</v>
       </c>
     </row>
     <row r="65">
@@ -2111,22 +2111,22 @@
         <v>62</v>
       </c>
       <c r="C65" t="n">
-        <v>0.4204853525649462</v>
+        <v>0.4187681562943192</v>
       </c>
       <c r="D65" t="n">
-        <v>0.1845636038217566</v>
+        <v>0.1739575303873617</v>
       </c>
       <c r="E65" t="n">
-        <v>0.3949510436132972</v>
+        <v>0.4072743133183191</v>
       </c>
       <c r="F65" t="n">
         <v>1</v>
       </c>
       <c r="G65" t="n">
-        <v>0.02553430895164899</v>
+        <v>0.01149384297600009</v>
       </c>
       <c r="H65" t="n">
-        <v>1.043060988852517</v>
+        <v>1.034595258201808</v>
       </c>
     </row>
     <row r="66">
@@ -2137,22 +2137,22 @@
         <v>61</v>
       </c>
       <c r="C66" t="n">
-        <v>0.4181625562603637</v>
+        <v>0.4165242509114151</v>
       </c>
       <c r="D66" t="n">
-        <v>0.1891598452346485</v>
+        <v>0.1784398548319403</v>
       </c>
       <c r="E66" t="n">
-        <v>0.3926775985049877</v>
+        <v>0.4050358942566446</v>
       </c>
       <c r="F66" t="n">
         <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>0.02548495775537601</v>
+        <v>0.01148835665477049</v>
       </c>
       <c r="H66" t="n">
-        <v>1.04663343399503</v>
+        <v>1.038401268941652</v>
       </c>
     </row>
     <row r="67">
@@ -2163,22 +2163,22 @@
         <v>60</v>
       </c>
       <c r="C67" t="n">
-        <v>0.4155962940541679</v>
+        <v>0.4140800948036308</v>
       </c>
       <c r="D67" t="n">
-        <v>0.1941081251809544</v>
+        <v>0.1832431290684501</v>
       </c>
       <c r="E67" t="n">
-        <v>0.3902955807648777</v>
+        <v>0.4026767761279191</v>
       </c>
       <c r="F67" t="n">
         <v>1</v>
       </c>
       <c r="G67" t="n">
-        <v>0.02530071328929012</v>
+        <v>0.01140331867571176</v>
       </c>
       <c r="H67" t="n">
-        <v>1.050329715701773</v>
+        <v>1.042328844982634</v>
       </c>
     </row>
     <row r="68">
@@ -2189,22 +2189,22 @@
         <v>59</v>
       </c>
       <c r="C68" t="n">
-        <v>0.4128786881794015</v>
+        <v>0.4114329448103516</v>
       </c>
       <c r="D68" t="n">
-        <v>0.1992373595135946</v>
+        <v>0.1882960309209064</v>
       </c>
       <c r="E68" t="n">
-        <v>0.3878839523070039</v>
+        <v>0.4002710242687419</v>
       </c>
       <c r="F68" t="n">
         <v>1</v>
       </c>
       <c r="G68" t="n">
-        <v>0.02499473587239759</v>
+        <v>0.01116192054160964</v>
       </c>
       <c r="H68" t="n">
-        <v>1.053999571573123</v>
+        <v>1.046296304541695</v>
       </c>
     </row>
     <row r="69">
@@ -2215,22 +2215,22 @@
         <v>58</v>
       </c>
       <c r="C69" t="n">
-        <v>0.4102499144579265</v>
+        <v>0.4088461443505979</v>
       </c>
       <c r="D69" t="n">
-        <v>0.2043962045639986</v>
+        <v>0.1934833476434879</v>
       </c>
       <c r="E69" t="n">
-        <v>0.3853538809780749</v>
+        <v>0.3976705080059142</v>
       </c>
       <c r="F69" t="n">
         <v>1</v>
       </c>
       <c r="G69" t="n">
-        <v>0.02489603347985159</v>
+        <v>0.0111756363446836</v>
       </c>
       <c r="H69" t="n">
-        <v>1.05751772717611</v>
+        <v>1.050191925647817</v>
       </c>
     </row>
     <row r="70">
@@ -2241,22 +2241,22 @@
         <v>57</v>
       </c>
       <c r="C70" t="n">
-        <v>0.4074204458716079</v>
+        <v>0.4060782952902676</v>
       </c>
       <c r="D70" t="n">
-        <v>0.2097491643197431</v>
+        <v>0.1988654287697199</v>
       </c>
       <c r="E70" t="n">
-        <v>0.382830389808649</v>
+        <v>0.3950562759400126</v>
       </c>
       <c r="F70" t="n">
         <v>1</v>
       </c>
       <c r="G70" t="n">
-        <v>0.02459005606295894</v>
+        <v>0.01102201935025499</v>
       </c>
       <c r="H70" t="n">
-        <v>1.061001634690476</v>
+        <v>1.054053888820583</v>
       </c>
     </row>
     <row r="71">
@@ -2267,22 +2267,22 @@
         <v>56</v>
       </c>
       <c r="C71" t="n">
-        <v>0.4045942673650409</v>
+        <v>0.4032775283025596</v>
       </c>
       <c r="D71" t="n">
-        <v>0.2151251546337483</v>
+        <v>0.2043215752325514</v>
       </c>
       <c r="E71" t="n">
-        <v>0.3802805780012107</v>
+        <v>0.3924008964648889</v>
       </c>
       <c r="F71" t="n">
         <v>1</v>
       </c>
       <c r="G71" t="n">
-        <v>0.02431368936383022</v>
+        <v>0.01087663183767074</v>
       </c>
       <c r="H71" t="n">
-        <v>1.064325549750122</v>
+        <v>1.05778325966735</v>
       </c>
     </row>
     <row r="72">
@@ -2293,22 +2293,22 @@
         <v>55</v>
       </c>
       <c r="C72" t="n">
-        <v>0.4016595162266733</v>
+        <v>0.4003286306416527</v>
       </c>
       <c r="D72" t="n">
-        <v>0.2207840918063854</v>
+        <v>0.2101096441297735</v>
       </c>
       <c r="E72" t="n">
-        <v>0.3775563919669413</v>
+        <v>0.3895617252285739</v>
       </c>
       <c r="F72" t="n">
         <v>1</v>
       </c>
       <c r="G72" t="n">
-        <v>0.02410312425973204</v>
+        <v>0.01076690541307884</v>
       </c>
       <c r="H72" t="n">
-        <v>1.067637032173546</v>
+        <v>1.061538791303916</v>
       </c>
     </row>
     <row r="73">
@@ -2319,22 +2319,22 @@
         <v>54</v>
       </c>
       <c r="C73" t="n">
-        <v>0.3986721238122812</v>
+        <v>0.3973824761413606</v>
       </c>
       <c r="D73" t="n">
-        <v>0.2266634643223752</v>
+        <v>0.2159772646848246</v>
       </c>
       <c r="E73" t="n">
-        <v>0.3746644118653436</v>
+        <v>0.3866402591738149</v>
       </c>
       <c r="F73" t="n">
         <v>1</v>
       </c>
       <c r="G73" t="n">
-        <v>0.02400771194693763</v>
+        <v>0.01074221696754568</v>
       </c>
       <c r="H73" t="n">
-        <v>1.070876555510471</v>
+        <v>1.065138712066902</v>
       </c>
     </row>
     <row r="74">
@@ -2345,22 +2345,22 @@
         <v>53</v>
       </c>
       <c r="C74" t="n">
-        <v>0.3955465480483247</v>
+        <v>0.3943430541801653</v>
       </c>
       <c r="D74" t="n">
-        <v>0.2325823177953834</v>
+        <v>0.2217927651881945</v>
       </c>
       <c r="E74" t="n">
-        <v>0.371871134156292</v>
+        <v>0.3838641806316402</v>
       </c>
       <c r="F74" t="n">
         <v>1</v>
       </c>
       <c r="G74" t="n">
-        <v>0.0236754138920327</v>
+        <v>0.01047887354852511</v>
       </c>
       <c r="H74" t="n">
-        <v>1.073945947171991</v>
+        <v>1.068509251848376</v>
       </c>
     </row>
     <row r="75">
@@ -2371,22 +2371,22 @@
         <v>52</v>
       </c>
       <c r="C75" t="n">
-        <v>0.3923716210880952</v>
+        <v>0.3911884194731486</v>
       </c>
       <c r="D75" t="n">
-        <v>0.2388367594030479</v>
+        <v>0.2280142534625545</v>
       </c>
       <c r="E75" t="n">
-        <v>0.3687916195088569</v>
+        <v>0.3807973270642969</v>
       </c>
       <c r="F75" t="n">
         <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>0.02358000157923829</v>
+        <v>0.01039109240885167</v>
       </c>
       <c r="H75" t="n">
-        <v>1.076968222581805</v>
+        <v>1.07189559183761</v>
       </c>
     </row>
     <row r="76">
@@ -2397,22 +2397,22 @@
         <v>51</v>
       </c>
       <c r="C76" t="n">
-        <v>0.3890848314163136</v>
+        <v>0.3879734352326063</v>
       </c>
       <c r="D76" t="n">
-        <v>0.2451109414892217</v>
+        <v>0.2343701566070395</v>
       </c>
       <c r="E76" t="n">
-        <v>0.3658042270944648</v>
+        <v>0.3776564081603542</v>
       </c>
       <c r="F76" t="n">
         <v>1</v>
       </c>
       <c r="G76" t="n">
-        <v>0.02328060432184881</v>
+        <v>0.01031702707225213</v>
       </c>
       <c r="H76" t="n">
-        <v>1.07979012199127</v>
+        <v>1.07512781832167</v>
       </c>
     </row>
     <row r="77">
@@ -2423,22 +2423,22 @@
         <v>50</v>
       </c>
       <c r="C77" t="n">
-        <v>0.3855578659226699</v>
+        <v>0.3845033370548879</v>
       </c>
       <c r="D77" t="n">
-        <v>0.2517667728265733</v>
+        <v>0.241030550579767</v>
       </c>
       <c r="E77" t="n">
-        <v>0.3626753612507567</v>
+        <v>0.3744661123653451</v>
       </c>
       <c r="F77" t="n">
         <v>1</v>
       </c>
       <c r="G77" t="n">
-        <v>0.02288250467191322</v>
+        <v>0.01003722468954282</v>
       </c>
       <c r="H77" t="n">
-        <v>1.082553629336951</v>
+        <v>1.078276073070528</v>
       </c>
     </row>
     <row r="78">
@@ -2449,22 +2449,22 @@
         <v>49</v>
       </c>
       <c r="C78" t="n">
-        <v>0.3819289079567288</v>
+        <v>0.3810030641104067</v>
       </c>
       <c r="D78" t="n">
-        <v>0.2588075434948543</v>
+        <v>0.2480310964687293</v>
       </c>
       <c r="E78" t="n">
-        <v>0.3592635485484168</v>
+        <v>0.3709658394208639</v>
       </c>
       <c r="F78" t="n">
         <v>1</v>
       </c>
       <c r="G78" t="n">
-        <v>0.02266535940831205</v>
+        <v>0.01003722468954282</v>
       </c>
       <c r="H78" t="n">
-        <v>1.085214801926697</v>
+        <v>1.08131985957876</v>
       </c>
     </row>
     <row r="79">
@@ -2475,22 +2475,22 @@
         <v>48</v>
       </c>
       <c r="C79" t="n">
-        <v>0.3782176979969994</v>
+        <v>0.3772778519955122</v>
       </c>
       <c r="D79" t="n">
-        <v>0.2660424288684758</v>
+        <v>0.2552318930825719</v>
       </c>
       <c r="E79" t="n">
-        <v>0.3557398731345248</v>
+        <v>0.3674902549219159</v>
       </c>
       <c r="F79" t="n">
         <v>1</v>
       </c>
       <c r="G79" t="n">
-        <v>0.02247782486247468</v>
+        <v>0.009787597073596221</v>
       </c>
       <c r="H79" t="n">
-        <v>1.087679061905591</v>
+        <v>1.084179903424149</v>
       </c>
     </row>
     <row r="80">
@@ -2501,22 +2501,22 @@
         <v>47</v>
       </c>
       <c r="C80" t="n">
-        <v>0.3743123733319296</v>
+        <v>0.373453886098485</v>
       </c>
       <c r="D80" t="n">
-        <v>0.2733661463953886</v>
+        <v>0.2626192246182206</v>
       </c>
       <c r="E80" t="n">
-        <v>0.3523214802726818</v>
+        <v>0.3639268892832944</v>
       </c>
       <c r="F80" t="n">
         <v>1</v>
       </c>
       <c r="G80" t="n">
-        <v>0.02199089305924778</v>
+        <v>0.009526996815190536</v>
       </c>
       <c r="H80" t="n">
-        <v>1.089909602103039</v>
+        <v>1.08683061010501</v>
       </c>
     </row>
     <row r="81">
@@ -2527,22 +2527,22 @@
         <v>46</v>
       </c>
       <c r="C81" t="n">
-        <v>0.3702622851577922</v>
+        <v>0.3694488716008811</v>
       </c>
       <c r="D81" t="n">
-        <v>0.2810155818177033</v>
+        <v>0.2703439649094894</v>
       </c>
       <c r="E81" t="n">
-        <v>0.3487221330245045</v>
+        <v>0.3602071634896295</v>
       </c>
       <c r="F81" t="n">
         <v>1</v>
       </c>
       <c r="G81" t="n">
-        <v>0.02154015213328775</v>
+        <v>0.009241708111251579</v>
       </c>
       <c r="H81" t="n">
-        <v>1.091949248187597</v>
+        <v>1.089301147270179</v>
       </c>
     </row>
     <row r="82">
@@ -2553,22 +2553,22 @@
         <v>45</v>
       </c>
       <c r="C82" t="n">
-        <v>0.366070723554339</v>
+        <v>0.3654219118183589</v>
       </c>
       <c r="D82" t="n">
-        <v>0.2888953228226252</v>
+        <v>0.2781372842161282</v>
       </c>
       <c r="E82" t="n">
-        <v>0.3450339536230358</v>
+        <v>0.356440803965513</v>
       </c>
       <c r="F82" t="n">
         <v>1</v>
       </c>
       <c r="G82" t="n">
-        <v>0.0210367699313031</v>
+        <v>0.008981107852845893</v>
       </c>
       <c r="H82" t="n">
-        <v>1.093748592591846</v>
+        <v>1.091486668959312</v>
       </c>
     </row>
     <row r="83">
@@ -2579,22 +2579,22 @@
         <v>44</v>
       </c>
       <c r="C83" t="n">
-        <v>0.3617541389203274</v>
+        <v>0.3611782423472677</v>
       </c>
       <c r="D83" t="n">
-        <v>0.2971271023609612</v>
+        <v>0.2863667660605196</v>
       </c>
       <c r="E83" t="n">
-        <v>0.3411187587187113</v>
+        <v>0.3524549915922127</v>
       </c>
       <c r="F83" t="n">
         <v>1</v>
       </c>
       <c r="G83" t="n">
-        <v>0.02063538020161609</v>
+        <v>0.008723250755054979</v>
       </c>
       <c r="H83" t="n">
-        <v>1.095301822261205</v>
+        <v>1.093465952171546</v>
       </c>
     </row>
     <row r="84">
@@ -2605,22 +2605,22 @@
         <v>43</v>
       </c>
       <c r="C84" t="n">
-        <v>0.3573783328507883</v>
+        <v>0.3569455455186357</v>
       </c>
       <c r="D84" t="n">
-        <v>0.3055135156476193</v>
+        <v>0.2945660731381483</v>
       </c>
       <c r="E84" t="n">
-        <v>0.3371081515015924</v>
+        <v>0.348488381343216</v>
       </c>
       <c r="F84" t="n">
         <v>1</v>
       </c>
       <c r="G84" t="n">
-        <v>0.02027018134919589</v>
+        <v>0.00845716417541964</v>
       </c>
       <c r="H84" t="n">
-        <v>1.096549251841696</v>
+        <v>1.09510843673517</v>
       </c>
     </row>
     <row r="85">
@@ -2631,22 +2631,22 @@
         <v>42</v>
       </c>
       <c r="C85" t="n">
-        <v>0.3529104045482063</v>
+        <v>0.3524851663589755</v>
       </c>
       <c r="D85" t="n">
-        <v>0.3139887610875687</v>
+        <v>0.3032070290747594</v>
       </c>
       <c r="E85" t="n">
-        <v>0.333100834364225</v>
+        <v>0.3443078045662651</v>
       </c>
       <c r="F85" t="n">
         <v>1</v>
       </c>
       <c r="G85" t="n">
-        <v>0.01980957018398127</v>
+        <v>0.008177361792710336</v>
       </c>
       <c r="H85" t="n">
-        <v>1.097475743733638</v>
+        <v>1.096489267808185</v>
       </c>
     </row>
     <row r="86">
@@ -2657,22 +2657,22 @@
         <v>41</v>
       </c>
       <c r="C86" t="n">
-        <v>0.3482878424973022</v>
+        <v>0.3479726671476341</v>
       </c>
       <c r="D86" t="n">
-        <v>0.3229739688890059</v>
+        <v>0.3122704317460492</v>
       </c>
       <c r="E86" t="n">
-        <v>0.328738188613692</v>
+        <v>0.3397569011063167</v>
       </c>
       <c r="F86" t="n">
         <v>1</v>
       </c>
       <c r="G86" t="n">
-        <v>0.01954965388361019</v>
+        <v>0.008215766041317463</v>
       </c>
       <c r="H86" t="n">
-        <v>1.098087248407208</v>
+        <v>1.097553980505716</v>
       </c>
     </row>
     <row r="87">
@@ -2683,22 +2683,22 @@
         <v>40</v>
       </c>
       <c r="C87" t="n">
-        <v>0.3432013792014318</v>
+        <v>0.343078868610836</v>
       </c>
       <c r="D87" t="n">
-        <v>0.3325152001684521</v>
+        <v>0.3217727401157065</v>
       </c>
       <c r="E87" t="n">
-        <v>0.3242834206301161</v>
+        <v>0.3351483912734575</v>
       </c>
       <c r="F87" t="n">
         <v>1</v>
       </c>
       <c r="G87" t="n">
-        <v>0.01891795857131578</v>
+        <v>0.007930477337378561</v>
       </c>
       <c r="H87" t="n">
-        <v>1.098342655258635</v>
+        <v>1.098263428625466</v>
       </c>
     </row>
     <row r="88">
@@ -2709,22 +2709,22 @@
         <v>39</v>
       </c>
       <c r="C88" t="n">
-        <v>0.3382465190956229</v>
+        <v>0.3381274637011272</v>
       </c>
       <c r="D88" t="n">
-        <v>0.3419675992946069</v>
+        <v>0.3314670697283997</v>
       </c>
       <c r="E88" t="n">
-        <v>0.3197858816097702</v>
+        <v>0.3304054665704731</v>
       </c>
       <c r="F88" t="n">
         <v>1</v>
       </c>
       <c r="G88" t="n">
-        <v>0.01846063748585264</v>
+        <v>0.007721997130654024</v>
       </c>
       <c r="H88" t="n">
-        <v>1.098186273097853</v>
+        <v>1.098559843633459</v>
       </c>
     </row>
     <row r="89">
@@ -2735,22 +2735,22 @@
         <v>38</v>
       </c>
       <c r="C89" t="n">
-        <v>0.3330975442844735</v>
+        <v>0.3329785512271529</v>
       </c>
       <c r="D89" t="n">
-        <v>0.3517259758376543</v>
+        <v>0.3415619007908532</v>
       </c>
       <c r="E89" t="n">
-        <v>0.3151764798778722</v>
+        <v>0.3254595479819939</v>
       </c>
       <c r="F89" t="n">
         <v>1</v>
       </c>
       <c r="G89" t="n">
-        <v>0.01792106440660124</v>
+        <v>0.007519003245159028</v>
       </c>
       <c r="H89" t="n">
-        <v>1.097610113577908</v>
+        <v>1.09841762263629</v>
       </c>
     </row>
     <row r="90">
@@ -2761,22 +2761,22 @@
         <v>37</v>
       </c>
       <c r="C90" t="n">
-        <v>0.3276722027741952</v>
+        <v>0.3274154215003443</v>
       </c>
       <c r="D90" t="n">
-        <v>0.3620008949016924</v>
+        <v>0.3522355387430289</v>
       </c>
       <c r="E90" t="n">
-        <v>0.3103269023241124</v>
+        <v>0.3203490397566268</v>
       </c>
       <c r="F90" t="n">
         <v>1</v>
       </c>
       <c r="G90" t="n">
-        <v>0.01734530045008287</v>
+        <v>0.007066381743717487</v>
       </c>
       <c r="H90" t="n">
-        <v>1.096552221908132</v>
+        <v>1.097777115179991</v>
       </c>
     </row>
     <row r="91">
@@ -2787,22 +2787,22 @@
         <v>36</v>
       </c>
       <c r="C91" t="n">
-        <v>0.3222172505461532</v>
+        <v>0.3219949361255051</v>
       </c>
       <c r="D91" t="n">
-        <v>0.3724238675545495</v>
+        <v>0.362958553586271</v>
       </c>
       <c r="E91" t="n">
-        <v>0.3053588818992972</v>
+        <v>0.3150465102882239</v>
       </c>
       <c r="F91" t="n">
         <v>1</v>
       </c>
       <c r="G91" t="n">
-        <v>0.01685836864685603</v>
+        <v>0.006948425837281169</v>
       </c>
       <c r="H91" t="n">
-        <v>1.095009279043882</v>
+        <v>1.096627052060483</v>
       </c>
     </row>
     <row r="92">
@@ -2813,22 +2813,22 @@
         <v>35</v>
       </c>
       <c r="C92" t="n">
-        <v>0.3162720764351328</v>
+        <v>0.3160395344307805</v>
       </c>
       <c r="D92" t="n">
-        <v>0.3834620851209433</v>
+        <v>0.3742411731949317</v>
       </c>
       <c r="E92" t="n">
-        <v>0.3002658384439239</v>
+        <v>0.3097192923742878</v>
       </c>
       <c r="F92" t="n">
         <v>1</v>
       </c>
       <c r="G92" t="n">
-        <v>0.01600623799120887</v>
+        <v>0.006320242056492675</v>
       </c>
       <c r="H92" t="n">
-        <v>1.092877294805363</v>
+        <v>1.094885426589823</v>
       </c>
     </row>
     <row r="93">
@@ -2839,22 +2839,22 @@
         <v>34</v>
       </c>
       <c r="C93" t="n">
-        <v>0.3101130471402627</v>
+        <v>0.3099497178659308</v>
       </c>
       <c r="D93" t="n">
-        <v>0.3951056773616192</v>
+        <v>0.3862095829572917</v>
       </c>
       <c r="E93" t="n">
-        <v>0.2947812754981181</v>
+        <v>0.3038406991767775</v>
       </c>
       <c r="F93" t="n">
         <v>1</v>
       </c>
       <c r="G93" t="n">
-        <v>0.01533177164214461</v>
+        <v>0.006109018689153312</v>
       </c>
       <c r="H93" t="n">
-        <v>1.090063685542828</v>
+        <v>1.092439047519332</v>
       </c>
     </row>
     <row r="94">
@@ -2865,22 +2865,22 @@
         <v>33</v>
       </c>
       <c r="C94" t="n">
-        <v>0.3036941015450215</v>
+        <v>0.3036404484518973</v>
       </c>
       <c r="D94" t="n">
-        <v>0.4070947279762062</v>
+        <v>0.3983782434445319</v>
       </c>
       <c r="E94" t="n">
-        <v>0.2892111704787724</v>
+        <v>0.2979813081035708</v>
       </c>
       <c r="F94" t="n">
         <v>1</v>
       </c>
       <c r="G94" t="n">
-        <v>0.01448293106624904</v>
+        <v>0.005659140348326541</v>
       </c>
       <c r="H94" t="n">
-        <v>1.086577378496151</v>
+        <v>1.089334424113648</v>
       </c>
     </row>
     <row r="95">
@@ -2891,22 +2891,22 @@
         <v>32</v>
       </c>
       <c r="C95" t="n">
-        <v>0.2969395678151238</v>
+        <v>0.2969553660336366</v>
       </c>
       <c r="D95" t="n">
-        <v>0.4198437870133972</v>
+        <v>0.4113369341888337</v>
       </c>
       <c r="E95" t="n">
-        <v>0.2832166451714789</v>
+        <v>0.2917076997775297</v>
       </c>
       <c r="F95" t="n">
         <v>1</v>
       </c>
       <c r="G95" t="n">
-        <v>0.01372292264364489</v>
+        <v>0.005247666256106953</v>
       </c>
       <c r="H95" t="n">
-        <v>1.08221285397256</v>
+        <v>1.085348201989514</v>
       </c>
     </row>
     <row r="96">
@@ -2917,22 +2917,22 @@
         <v>31</v>
       </c>
       <c r="C96" t="n">
-        <v>0.2900600110546679</v>
+        <v>0.2899465906628299</v>
       </c>
       <c r="D96" t="n">
-        <v>0.4328231516331956</v>
+        <v>0.4246412631705999</v>
       </c>
       <c r="E96" t="n">
-        <v>0.2771168373121364</v>
+        <v>0.2854121461665702</v>
       </c>
       <c r="F96" t="n">
         <v>1</v>
       </c>
       <c r="G96" t="n">
-        <v>0.01294317374253151</v>
+        <v>0.004534444496259726</v>
       </c>
       <c r="H96" t="n">
-        <v>1.077083705342805</v>
+        <v>1.080536321034866</v>
       </c>
     </row>
     <row r="97">
@@ -2943,22 +2943,22 @@
         <v>30</v>
       </c>
       <c r="C97" t="n">
-        <v>0.2829369883925986</v>
+        <v>0.2829405584526379</v>
       </c>
       <c r="D97" t="n">
-        <v>0.4464309214855368</v>
+        <v>0.4385490874876215</v>
       </c>
       <c r="E97" t="n">
-        <v>0.2706320901218646</v>
+        <v>0.2785103540597406</v>
       </c>
       <c r="F97" t="n">
         <v>1</v>
       </c>
       <c r="G97" t="n">
-        <v>0.01230489827073405</v>
+        <v>0.004430204392897374</v>
       </c>
       <c r="H97" t="n">
-        <v>1.070964930945571</v>
+        <v>1.07472625767152</v>
       </c>
     </row>
     <row r="98">
@@ -2969,22 +2969,22 @@
         <v>29</v>
       </c>
       <c r="C98" t="n">
-        <v>0.2754290263995999</v>
+        <v>0.275555970077604</v>
       </c>
       <c r="D98" t="n">
-        <v>0.4605716842576264</v>
+        <v>0.4528409542907147</v>
       </c>
       <c r="E98" t="n">
-        <v>0.2639992893427737</v>
+        <v>0.2716030756316813</v>
       </c>
       <c r="F98" t="n">
         <v>1</v>
       </c>
       <c r="G98" t="n">
-        <v>0.01142973705682626</v>
+        <v>0.003952894445922728</v>
       </c>
       <c r="H98" t="n">
-        <v>1.063816879990652</v>
+        <v>1.067940079126627</v>
       </c>
     </row>
     <row r="99">
@@ -2995,22 +2995,22 @@
         <v>28</v>
       </c>
       <c r="C99" t="n">
-        <v>0.2679868660016319</v>
+        <v>0.2680451963142894</v>
       </c>
       <c r="D99" t="n">
-        <v>0.4749855236490932</v>
+        <v>0.4678487860142699</v>
       </c>
       <c r="E99" t="n">
-        <v>0.2570276103492748</v>
+        <v>0.2641060176714407</v>
       </c>
       <c r="F99" t="n">
         <v>1</v>
       </c>
       <c r="G99" t="n">
-        <v>0.01095925565235706</v>
+        <v>0.003939178642848706</v>
       </c>
       <c r="H99" t="n">
-        <v>1.055693119838059</v>
+        <v>1.059922883210434</v>
       </c>
     </row>
     <row r="100">
@@ -3021,22 +3021,22 @@
         <v>27</v>
       </c>
       <c r="C100" t="n">
-        <v>0.2600939646777038</v>
+        <v>0.2599720746249414</v>
       </c>
       <c r="D100" t="n">
-        <v>0.490281104413971</v>
+        <v>0.4834875446792285</v>
       </c>
       <c r="E100" t="n">
-        <v>0.2496249309083252</v>
+        <v>0.2565403806958301</v>
       </c>
       <c r="F100" t="n">
         <v>1</v>
       </c>
       <c r="G100" t="n">
-        <v>0.01046903376937858</v>
+        <v>0.003431693929111246</v>
       </c>
       <c r="H100" t="n">
-        <v>1.046160948698919</v>
+        <v>1.05060950803757</v>
       </c>
     </row>
     <row r="101">
@@ -3047,22 +3047,22 @@
         <v>26</v>
       </c>
       <c r="C101" t="n">
-        <v>0.2520135288079383</v>
+        <v>0.2517892265110014</v>
       </c>
       <c r="D101" t="n">
-        <v>0.5059649145895296</v>
+        <v>0.4995706953637842</v>
       </c>
       <c r="E101" t="n">
-        <v>0.2420215566025321</v>
+        <v>0.2486400781252143</v>
       </c>
       <c r="F101" t="n">
         <v>1</v>
       </c>
       <c r="G101" t="n">
-        <v>0.009991972205406263</v>
+        <v>0.003149148385787143</v>
       </c>
       <c r="H101" t="n">
-        <v>1.035413990162082</v>
+        <v>1.040008061839811</v>
       </c>
     </row>
     <row r="102">
@@ -3073,22 +3073,22 @@
         <v>25</v>
       </c>
       <c r="C102" t="n">
-        <v>0.2432981075461269</v>
+        <v>0.2432168495897603</v>
       </c>
       <c r="D102" t="n">
-        <v>0.5224712447029716</v>
+        <v>0.5161037243891667</v>
       </c>
       <c r="E102" t="n">
-        <v>0.2342306477509015</v>
+        <v>0.240679426021073</v>
       </c>
       <c r="F102" t="n">
         <v>1</v>
       </c>
       <c r="G102" t="n">
-        <v>0.009067459795225413</v>
+        <v>0.002537423568687386</v>
       </c>
       <c r="H102" t="n">
-        <v>1.023048541000749</v>
+        <v>1.02803311427989</v>
       </c>
     </row>
     <row r="103">
@@ -3099,22 +3099,22 @@
         <v>24</v>
       </c>
       <c r="C103" t="n">
-        <v>0.2344576632537573</v>
+        <v>0.2345621778500753</v>
       </c>
       <c r="D103" t="n">
-        <v>0.5393329034295792</v>
+        <v>0.5330399980249244</v>
       </c>
       <c r="E103" t="n">
-        <v>0.2262094333166636</v>
+        <v>0.2323978241250003</v>
       </c>
       <c r="F103" t="n">
         <v>1</v>
       </c>
       <c r="G103" t="n">
-        <v>0.008248229937093676</v>
+        <v>0.002164353725074952</v>
       </c>
       <c r="H103" t="n">
-        <v>1.009286076854825</v>
+        <v>1.014629295840312</v>
       </c>
     </row>
     <row r="104">
@@ -3125,22 +3125,22 @@
         <v>23</v>
       </c>
       <c r="C104" t="n">
-        <v>0.2254263943357987</v>
+        <v>0.2255316931061631</v>
       </c>
       <c r="D104" t="n">
-        <v>0.5568624483457479</v>
+        <v>0.5508239082906543</v>
       </c>
       <c r="E104" t="n">
-        <v>0.2177111573184534</v>
+        <v>0.2236443986031826</v>
       </c>
       <c r="F104" t="n">
         <v>1</v>
       </c>
       <c r="G104" t="n">
-        <v>0.007715237017345306</v>
+        <v>0.001887294502980447</v>
       </c>
       <c r="H104" t="n">
-        <v>0.9937588677299642</v>
+        <v>0.9993132815748889</v>
       </c>
     </row>
     <row r="105">
@@ -3151,22 +3151,22 @@
         <v>22</v>
       </c>
       <c r="C105" t="n">
-        <v>0.2161384991972205</v>
+        <v>0.2160540731820389</v>
       </c>
       <c r="D105" t="n">
-        <v>0.5748986655436528</v>
+        <v>0.5692387454977876</v>
       </c>
       <c r="E105" t="n">
-        <v>0.2089628352591267</v>
+        <v>0.2147071813201735</v>
       </c>
       <c r="F105" t="n">
         <v>1</v>
       </c>
       <c r="G105" t="n">
-        <v>0.007175663938093851</v>
+        <v>0.001346891861865401</v>
       </c>
       <c r="H105" t="n">
-        <v>0.9764824425328764</v>
+        <v>0.9821071323537554</v>
       </c>
     </row>
     <row r="106">
@@ -3177,22 +3177,22 @@
         <v>21</v>
       </c>
       <c r="C106" t="n">
-        <v>0.2063998631326823</v>
+        <v>0.2061238317564732</v>
       </c>
       <c r="D106" t="n">
-        <v>0.5934086542257785</v>
+        <v>0.5883064549312427</v>
       </c>
       <c r="E106" t="n">
-        <v>0.2001914826415392</v>
+        <v>0.2055697133122842</v>
       </c>
       <c r="F106" t="n">
         <v>1</v>
       </c>
       <c r="G106" t="n">
-        <v>0.006208380491143084</v>
+        <v>0.0005541184441890112</v>
       </c>
       <c r="H106" t="n">
-        <v>0.9573741193188396</v>
+        <v>0.9628328568275604</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Run-ready: experimental stack incl. JSON logging, blends, sizing polish
</commit_message>
<xml_diff>
--- a/figures/holding_period_scan_tp5_sl5.xlsx
+++ b/figures/holding_period_scan_tp5_sl5.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,2732 +467,2758 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B2" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4803630847389745</v>
+        <v>0.4831511955171277</v>
       </c>
       <c r="D2" t="n">
-        <v>0.05580960270804816</v>
+        <v>0.05710844595451203</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4638273125529773</v>
+        <v>0.4597403585283603</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.01653577218599728</v>
+        <v>0.02341083698876745</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8695964152627146</v>
+        <v>0.8722080020912304</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B3" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4799817854135178</v>
+        <v>0.4827784680138949</v>
       </c>
       <c r="D3" t="n">
-        <v>0.05651185182543623</v>
+        <v>0.0577296584599001</v>
       </c>
       <c r="E3" t="n">
-        <v>0.463506362761046</v>
+        <v>0.459491873526205</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01647542265247176</v>
+        <v>0.02328659448768988</v>
       </c>
       <c r="H3" t="n">
-        <v>0.8710921690580786</v>
+        <v>0.8735186061912252</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B4" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4796279176942089</v>
+        <v>0.4823905271431831</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0572195872640539</v>
+        <v>0.05845229341514744</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4631524950417372</v>
+        <v>0.4591571794416694</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0.01647542265247176</v>
+        <v>0.02323334770151375</v>
       </c>
       <c r="H4" t="n">
-        <v>0.8725891870708968</v>
+        <v>0.8750320007527035</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B5" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4792795362961297</v>
+        <v>0.4820330130074292</v>
       </c>
       <c r="D5" t="n">
-        <v>0.057894404775294</v>
+        <v>0.05916478612540886</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4628260589285763</v>
+        <v>0.4588022008671619</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0.01645347736755337</v>
+        <v>0.02323081214026723</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8740083106448806</v>
+        <v>0.8765136304420733</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B6" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4789119527737469</v>
+        <v>0.4816450721367175</v>
       </c>
       <c r="D6" t="n">
-        <v>0.05863505814128923</v>
+        <v>0.05988488551940972</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4624529890849639</v>
+        <v>0.4584700423438728</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0.01645896368878297</v>
+        <v>0.02317502979284464</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8755557611417806</v>
+        <v>0.8780031255247061</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B7" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C7" t="n">
-        <v>0.4785087081633717</v>
+        <v>0.4812520601435128</v>
       </c>
       <c r="D7" t="n">
-        <v>0.05937845466789926</v>
+        <v>0.06066076726083319</v>
       </c>
       <c r="E7" t="n">
-        <v>0.4621128371687291</v>
+        <v>0.4580871725956541</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>0.01639587099464257</v>
+        <v>0.02316488754785873</v>
       </c>
       <c r="H7" t="n">
-        <v>0.877100147200546</v>
+        <v>0.8795964655927141</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B8" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C8" t="n">
-        <v>0.4781219225166853</v>
+        <v>0.4808235502928573</v>
       </c>
       <c r="D8" t="n">
-        <v>0.06014379647942766</v>
+        <v>0.06141890007353128</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4617342810038871</v>
+        <v>0.4577575496336114</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0163876415127982</v>
+        <v>0.02306600065924591</v>
       </c>
       <c r="H8" t="n">
-        <v>0.8786787976294317</v>
+        <v>0.8811453416986768</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B9" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C9" t="n">
-        <v>0.4776610715333994</v>
+        <v>0.4804305382996527</v>
       </c>
       <c r="D9" t="n">
-        <v>0.06095851518202242</v>
+        <v>0.06220238849869419</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4613804132845782</v>
+        <v>0.4573670732016532</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>0.01628065824882113</v>
+        <v>0.02306346509799945</v>
       </c>
       <c r="H9" t="n">
-        <v>0.8803496205677421</v>
+        <v>0.8827330911695535</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B10" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C10" t="n">
-        <v>0.4772303953168762</v>
+        <v>0.4799690661527929</v>
       </c>
       <c r="D10" t="n">
-        <v>0.06178146336646157</v>
+        <v>0.06302137478130784</v>
       </c>
       <c r="E10" t="n">
-        <v>0.4609881413166622</v>
+        <v>0.4570095590658992</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0.01624225400021401</v>
+        <v>0.0229595070868937</v>
       </c>
       <c r="H10" t="n">
-        <v>0.8820243359120739</v>
+        <v>0.8843840180906657</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B11" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C11" t="n">
-        <v>0.4767914896185086</v>
+        <v>0.479532949618398</v>
       </c>
       <c r="D11" t="n">
-        <v>0.06267024740565585</v>
+        <v>0.06384036106392151</v>
       </c>
       <c r="E11" t="n">
-        <v>0.4605382629758355</v>
+        <v>0.4566266893176805</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>0.01625322664267315</v>
+        <v>0.02290626030071757</v>
       </c>
       <c r="H11" t="n">
-        <v>0.8838190004514528</v>
+        <v>0.8860223386196107</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B12" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C12" t="n">
-        <v>0.4763498407595263</v>
+        <v>0.4790968330840031</v>
       </c>
       <c r="D12" t="n">
-        <v>0.06353708615993175</v>
+        <v>0.06471512969395776</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4601130730805419</v>
+        <v>0.4561880372220391</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0.01623676767898435</v>
+        <v>0.02290879586196404</v>
       </c>
       <c r="H12" t="n">
-        <v>0.8855568676679775</v>
+        <v>0.887758400072821</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B13" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C13" t="n">
-        <v>0.4759465961491511</v>
+        <v>0.4786505743046223</v>
       </c>
       <c r="D13" t="n">
-        <v>0.06440118175359286</v>
+        <v>0.06557975607900809</v>
       </c>
       <c r="E13" t="n">
-        <v>0.459652222097256</v>
+        <v>0.4557696696163696</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0162943740518951</v>
+        <v>0.02288090468825271</v>
       </c>
       <c r="H13" t="n">
-        <v>0.8872753797340196</v>
+        <v>0.8894626531086438</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B14" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C14" t="n">
-        <v>0.475543351538776</v>
+        <v>0.4782423489439387</v>
       </c>
       <c r="D14" t="n">
-        <v>0.06520767097434321</v>
+        <v>0.06643677578031898</v>
       </c>
       <c r="E14" t="n">
-        <v>0.4592489774868808</v>
+        <v>0.4553208752757423</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>0.01629437405189516</v>
+        <v>0.02292147366819647</v>
       </c>
       <c r="H14" t="n">
-        <v>0.8888690743711101</v>
+        <v>0.8911382001519901</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B15" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C15" t="n">
-        <v>0.47508250055549</v>
+        <v>0.4778315880220086</v>
       </c>
       <c r="D15" t="n">
-        <v>0.06604433496185635</v>
+        <v>0.0672456198179467</v>
       </c>
       <c r="E15" t="n">
-        <v>0.4588731644826536</v>
+        <v>0.4549227921600446</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>0.01620933607283637</v>
+        <v>0.02290879586196404</v>
       </c>
       <c r="H15" t="n">
-        <v>0.8905126012727143</v>
+        <v>0.8927099442937257</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B16" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C16" t="n">
-        <v>0.4746024474479005</v>
+        <v>0.4773701158751489</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0669605506071986</v>
+        <v>0.06809249727427166</v>
       </c>
       <c r="E16" t="n">
-        <v>0.4584370019449009</v>
+        <v>0.4545373868505794</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>0.01616544550299964</v>
+        <v>0.02283272902456956</v>
       </c>
       <c r="H16" t="n">
-        <v>0.8922985261471452</v>
+        <v>0.8943459599012977</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B17" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C17" t="n">
-        <v>0.4741141648584666</v>
+        <v>0.476875681432085</v>
       </c>
       <c r="D17" t="n">
-        <v>0.06787950941315565</v>
+        <v>0.06902304825173051</v>
       </c>
       <c r="E17" t="n">
-        <v>0.4580063257283777</v>
+        <v>0.4541012703161845</v>
       </c>
       <c r="F17" t="n">
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0161078391300889</v>
+        <v>0.02277441111590051</v>
       </c>
       <c r="H17" t="n">
-        <v>0.8940765353057702</v>
+        <v>0.8961299681831969</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B18" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C18" t="n">
-        <v>0.4736203959478031</v>
+        <v>0.4763837825502675</v>
       </c>
       <c r="D18" t="n">
-        <v>0.06884235878894945</v>
+        <v>0.06994345698420346</v>
       </c>
       <c r="E18" t="n">
-        <v>0.4575372452632474</v>
+        <v>0.4536727604655291</v>
       </c>
       <c r="F18" t="n">
         <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>0.01608315068455574</v>
+        <v>0.02271102208473841</v>
       </c>
       <c r="H18" t="n">
-        <v>0.8959245309190129</v>
+        <v>0.8978814132580664</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B19" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C19" t="n">
-        <v>0.4730553048611549</v>
+        <v>0.4758715991784782</v>
       </c>
       <c r="D19" t="n">
-        <v>0.06992042091056473</v>
+        <v>0.07093739699282436</v>
       </c>
       <c r="E19" t="n">
-        <v>0.4570242742282803</v>
+        <v>0.4531910038286975</v>
       </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>0.01603103063287459</v>
+        <v>0.02268059534978067</v>
       </c>
       <c r="H19" t="n">
-        <v>0.8979769230186758</v>
+        <v>0.8997572305495811</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B20" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C20" t="n">
-        <v>0.4725149022200399</v>
+        <v>0.4752934912142803</v>
       </c>
       <c r="D20" t="n">
-        <v>0.07095184930172846</v>
+        <v>0.07202008164507213</v>
       </c>
       <c r="E20" t="n">
-        <v>0.4565332484782316</v>
+        <v>0.4526864271406476</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0.01598165374180827</v>
+        <v>0.02260706407363267</v>
       </c>
       <c r="H20" t="n">
-        <v>0.8999237925166172</v>
+        <v>0.9017844651900868</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B21" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C21" t="n">
-        <v>0.4719168932060141</v>
+        <v>0.4747356677400543</v>
       </c>
       <c r="D21" t="n">
-        <v>0.07209026095686928</v>
+        <v>0.07306726843986916</v>
       </c>
       <c r="E21" t="n">
-        <v>0.4559928458371166</v>
+        <v>0.4521970638200766</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>0.01592404736889746</v>
+        <v>0.0225386039199777</v>
       </c>
       <c r="H21" t="n">
-        <v>0.902053921270815</v>
+        <v>0.9037284769321112</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B22" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C22" t="n">
-        <v>0.4713490589587511</v>
+        <v>0.4741169907959127</v>
       </c>
       <c r="D22" t="n">
-        <v>0.07317380939971416</v>
+        <v>0.07422348436826491</v>
       </c>
       <c r="E22" t="n">
-        <v>0.4554771316415347</v>
+        <v>0.4516595248358224</v>
       </c>
       <c r="F22" t="n">
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>0.01587192731721637</v>
+        <v>0.02245746596009029</v>
       </c>
       <c r="H22" t="n">
-        <v>0.9040633446357331</v>
+        <v>0.9058562246134435</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B23" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C23" t="n">
-        <v>0.4707976836751769</v>
+        <v>0.4735287405867289</v>
       </c>
       <c r="D23" t="n">
-        <v>0.07423541255764066</v>
+        <v>0.07533152463297751</v>
       </c>
       <c r="E23" t="n">
-        <v>0.4549669037671825</v>
+        <v>0.4511397347802936</v>
       </c>
       <c r="F23" t="n">
         <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>0.01583077990799442</v>
+        <v>0.02238900580643527</v>
       </c>
       <c r="H23" t="n">
-        <v>0.9060151085476411</v>
+        <v>0.9078768279703715</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B24" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C24" t="n">
-        <v>0.4701996746611511</v>
+        <v>0.4729810593574888</v>
       </c>
       <c r="D24" t="n">
-        <v>0.07537931053401108</v>
+        <v>0.07639392479525343</v>
       </c>
       <c r="E24" t="n">
-        <v>0.4544210148048378</v>
+        <v>0.4506250158472578</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>0.01577865985631327</v>
+        <v>0.02235604351023102</v>
       </c>
       <c r="H24" t="n">
-        <v>0.908099954884276</v>
+        <v>0.9097968551767084</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B25" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C25" t="n">
-        <v>0.4696236109320437</v>
+        <v>0.4723674535358401</v>
       </c>
       <c r="D25" t="n">
-        <v>0.07656161275898865</v>
+        <v>0.07755014072364919</v>
       </c>
       <c r="E25" t="n">
-        <v>0.4538147763089677</v>
+        <v>0.4500824057405107</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0.01580883462307603</v>
+        <v>0.02228504779532947</v>
       </c>
       <c r="H25" t="n">
-        <v>0.910233631961729</v>
+        <v>0.9118691088647676</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B26" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C26" t="n">
-        <v>0.4689323344571148</v>
+        <v>0.4717918811328888</v>
       </c>
       <c r="D26" t="n">
-        <v>0.07779603503564737</v>
+        <v>0.07872410558077031</v>
       </c>
       <c r="E26" t="n">
-        <v>0.4532716305072378</v>
+        <v>0.4494840132863409</v>
       </c>
       <c r="F26" t="n">
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>0.01566070394987695</v>
+        <v>0.02230786784654787</v>
       </c>
       <c r="H26" t="n">
-        <v>0.9124433399969795</v>
+        <v>0.9139517584018364</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B27" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C27" t="n">
-        <v>0.4682849485520227</v>
+        <v>0.4710996729125992</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0790139983486173</v>
+        <v>0.079958923907807</v>
       </c>
       <c r="E27" t="n">
-        <v>0.45270105309936</v>
+        <v>0.4489414031795938</v>
       </c>
       <c r="F27" t="n">
         <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>0.01558389545266264</v>
+        <v>0.02215826973300539</v>
       </c>
       <c r="H27" t="n">
-        <v>0.9146015784738277</v>
+        <v>0.9161260574342791</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B28" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C28" t="n">
-        <v>0.4675717267921754</v>
+        <v>0.4704353558660209</v>
       </c>
       <c r="D28" t="n">
-        <v>0.08026487958896482</v>
+        <v>0.08119627779609016</v>
       </c>
       <c r="E28" t="n">
-        <v>0.4521633936188598</v>
+        <v>0.4483683663378889</v>
       </c>
       <c r="F28" t="n">
         <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>0.01540833317331564</v>
+        <v>0.02206698952813202</v>
       </c>
       <c r="H28" t="n">
-        <v>0.9167985520326524</v>
+        <v>0.918282607838901</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B29" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C29" t="n">
-        <v>0.4668310734261802</v>
+        <v>0.469720327594513</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0816254872539042</v>
+        <v>0.08243616724561982</v>
       </c>
       <c r="E29" t="n">
-        <v>0.4515434393199156</v>
+        <v>0.4478435051598672</v>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>0.01528763410626455</v>
+        <v>0.02187682243464589</v>
       </c>
       <c r="H29" t="n">
-        <v>0.9191629890890132</v>
+        <v>0.9204253461490386</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B30" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C30" t="n">
-        <v>0.4660547589721926</v>
+        <v>0.4689748725880474</v>
       </c>
       <c r="D30" t="n">
-        <v>0.08303272864929515</v>
+        <v>0.08380029919622708</v>
       </c>
       <c r="E30" t="n">
-        <v>0.4509125123785123</v>
+        <v>0.4472248282157256</v>
       </c>
       <c r="F30" t="n">
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0151422465936803</v>
+        <v>0.02175004437232181</v>
       </c>
       <c r="H30" t="n">
-        <v>0.9215828175278882</v>
+        <v>0.922757338954683</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B31" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C31" t="n">
-        <v>0.4652757013575902</v>
+        <v>0.4682116686528563</v>
       </c>
       <c r="D31" t="n">
-        <v>0.08449483325698202</v>
+        <v>0.08520246456553159</v>
       </c>
       <c r="E31" t="n">
-        <v>0.4502294653854278</v>
+        <v>0.4465858667816121</v>
       </c>
       <c r="F31" t="n">
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>0.01504623597216237</v>
+        <v>0.02162580187124419</v>
       </c>
       <c r="H31" t="n">
-        <v>0.9240685197698018</v>
+        <v>0.9251289389738462</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B32" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C32" t="n">
-        <v>0.4645323048309802</v>
+        <v>0.4674433935951723</v>
       </c>
       <c r="D32" t="n">
-        <v>0.08589658833114337</v>
+        <v>0.08665534115976571</v>
       </c>
       <c r="E32" t="n">
-        <v>0.4495711068378765</v>
+        <v>0.445901265245062</v>
       </c>
       <c r="F32" t="n">
         <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>0.01496119799310369</v>
+        <v>0.02154212835011027</v>
       </c>
       <c r="H32" t="n">
-        <v>0.9264255479521235</v>
+        <v>0.9275586339535722</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B33" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C33" t="n">
-        <v>0.4637395314133038</v>
+        <v>0.466710616394939</v>
       </c>
       <c r="D33" t="n">
-        <v>0.08744921723911857</v>
+        <v>0.08805497096782373</v>
       </c>
       <c r="E33" t="n">
-        <v>0.4488112513475777</v>
+        <v>0.4452344126372372</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>0.01492828006572611</v>
+        <v>0.02147620375770176</v>
       </c>
       <c r="H33" t="n">
-        <v>0.9290060667504286</v>
+        <v>0.9298737065439595</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B34" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C34" t="n">
-        <v>0.4629056105864054</v>
+        <v>0.4658967012348183</v>
       </c>
       <c r="D34" t="n">
-        <v>0.08910059992922646</v>
+        <v>0.08963716118562844</v>
       </c>
       <c r="E34" t="n">
-        <v>0.4479937894843681</v>
+        <v>0.4444661375795532</v>
       </c>
       <c r="F34" t="n">
         <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>0.01491182110203737</v>
+        <v>0.02143056365526508</v>
       </c>
       <c r="H34" t="n">
-        <v>0.9317172722827494</v>
+        <v>0.9324607054789653</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B35" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C35" t="n">
-        <v>0.4620579739564331</v>
+        <v>0.4650574304622328</v>
       </c>
       <c r="D35" t="n">
-        <v>0.09076569842240834</v>
+        <v>0.09126499150586982</v>
       </c>
       <c r="E35" t="n">
-        <v>0.4471763276211586</v>
+        <v>0.4436775780318973</v>
       </c>
       <c r="F35" t="n">
         <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>0.01488164633527456</v>
+        <v>0.02137985243033547</v>
       </c>
       <c r="H35" t="n">
-        <v>0.9344171980011662</v>
+        <v>0.9350904037279019</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B36" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C36" t="n">
-        <v>0.4611527309535501</v>
+        <v>0.4642384441796192</v>
       </c>
       <c r="D36" t="n">
-        <v>0.09246371484296777</v>
+        <v>0.09289282182611121</v>
       </c>
       <c r="E36" t="n">
-        <v>0.4463835542034822</v>
+        <v>0.4428687339942696</v>
       </c>
       <c r="F36" t="n">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>0.01476917675006789</v>
+        <v>0.02136971018534956</v>
       </c>
       <c r="H36" t="n">
-        <v>0.9371372364164533</v>
+        <v>0.9376871948331416</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B37" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C37" t="n">
-        <v>0.4602502311112818</v>
+        <v>0.4633332488146251</v>
       </c>
       <c r="D37" t="n">
-        <v>0.09424951240320072</v>
+        <v>0.0946043256674865</v>
       </c>
       <c r="E37" t="n">
-        <v>0.4455002564855175</v>
+        <v>0.4420624255178884</v>
       </c>
       <c r="F37" t="n">
         <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>0.01474997462576427</v>
+        <v>0.02127082329673674</v>
       </c>
       <c r="H37" t="n">
-        <v>0.9399592125075619</v>
+        <v>0.9403856366743099</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B38" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C38" t="n">
-        <v>0.4592901248961028</v>
+        <v>0.4624280534496311</v>
       </c>
       <c r="D38" t="n">
-        <v>0.09606822789081124</v>
+        <v>0.09639189634625625</v>
       </c>
       <c r="E38" t="n">
-        <v>0.444641647213086</v>
+        <v>0.4411800502041127</v>
       </c>
       <c r="F38" t="n">
         <v>1</v>
       </c>
       <c r="G38" t="n">
-        <v>0.0146484776830168</v>
+        <v>0.0212480032455184</v>
       </c>
       <c r="H38" t="n">
-        <v>0.94279614338955</v>
+        <v>0.9431656111669388</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B39" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C39" t="n">
-        <v>0.4583327618415386</v>
+        <v>0.4614696112984609</v>
       </c>
       <c r="D39" t="n">
-        <v>0.09790614550272533</v>
+        <v>0.09821750044372322</v>
       </c>
       <c r="E39" t="n">
-        <v>0.4437610926557361</v>
+        <v>0.4403128882578159</v>
       </c>
       <c r="F39" t="n">
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>0.01457166918580249</v>
+        <v>0.02115672304064503</v>
       </c>
       <c r="H39" t="n">
-        <v>0.9456239097315409</v>
+        <v>0.9459684680753481</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B40" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C40" t="n">
-        <v>0.4574467209629591</v>
+        <v>0.4605162402697837</v>
       </c>
       <c r="D40" t="n">
-        <v>0.09974131995402463</v>
+        <v>0.1000557823474226</v>
       </c>
       <c r="E40" t="n">
-        <v>0.4428119590830163</v>
+        <v>0.4394279773827937</v>
       </c>
       <c r="F40" t="n">
         <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>0.01463476187994278</v>
+        <v>0.02108826288699006</v>
       </c>
       <c r="H40" t="n">
-        <v>0.9484070281893636</v>
+        <v>0.9487522148529373</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B41" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C41" t="n">
-        <v>0.4564427241779433</v>
+        <v>0.459633864956008</v>
       </c>
       <c r="D41" t="n">
-        <v>0.101738340881597</v>
+        <v>0.1019118131798474</v>
       </c>
       <c r="E41" t="n">
-        <v>0.4418189349404597</v>
+        <v>0.4384543218641446</v>
       </c>
       <c r="F41" t="n">
         <v>1</v>
       </c>
       <c r="G41" t="n">
-        <v>0.01462378923748364</v>
+        <v>0.02117954309186337</v>
       </c>
       <c r="H41" t="n">
-        <v>0.9513942862675231</v>
+        <v>0.9515209951844967</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B42" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C42" t="n">
-        <v>0.4553728915381725</v>
+        <v>0.4586272471411547</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1036777554362586</v>
+        <v>0.1039225132483075</v>
       </c>
       <c r="E42" t="n">
-        <v>0.440949353025569</v>
+        <v>0.4374502396105378</v>
       </c>
       <c r="F42" t="n">
         <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>0.01442353851260347</v>
+        <v>0.02117700753061691</v>
       </c>
       <c r="H42" t="n">
-        <v>0.9542566656558367</v>
+        <v>0.9544804306642671</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B43" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C43" t="n">
-        <v>0.4543634084319271</v>
+        <v>0.4575825959076041</v>
       </c>
       <c r="D43" t="n">
-        <v>0.1056665468819865</v>
+        <v>0.1058393975506478</v>
       </c>
       <c r="E43" t="n">
-        <v>0.4399700446860864</v>
+        <v>0.436578006541748</v>
       </c>
       <c r="F43" t="n">
         <v>1</v>
       </c>
       <c r="G43" t="n">
-        <v>0.01439336374584066</v>
+        <v>0.02100458936585614</v>
       </c>
       <c r="H43" t="n">
-        <v>0.9571470542349066</v>
+        <v>0.9572653556669976</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B44" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C44" t="n">
-        <v>0.453323750558919</v>
+        <v>0.4565709069702579</v>
       </c>
       <c r="D44" t="n">
-        <v>0.1077623215916915</v>
+        <v>0.1078222064453967</v>
       </c>
       <c r="E44" t="n">
-        <v>0.4389139278493895</v>
+        <v>0.4356068865843454</v>
       </c>
       <c r="F44" t="n">
         <v>1</v>
       </c>
       <c r="G44" t="n">
-        <v>0.01440982270952951</v>
+        <v>0.02096402038591244</v>
       </c>
       <c r="H44" t="n">
-        <v>0.9601468663977858</v>
+        <v>0.9601019649120672</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B45" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C45" t="n">
-        <v>0.4521387051733266</v>
+        <v>0.4555338624204467</v>
       </c>
       <c r="D45" t="n">
-        <v>0.1100117132958252</v>
+        <v>0.1099470067699485</v>
       </c>
       <c r="E45" t="n">
-        <v>0.4378495815308482</v>
+        <v>0.4345191308096047</v>
       </c>
       <c r="F45" t="n">
         <v>1</v>
       </c>
       <c r="G45" t="n">
-        <v>0.01428912364247842</v>
+        <v>0.02101473161084205</v>
       </c>
       <c r="H45" t="n">
-        <v>0.9633179805749402</v>
+        <v>0.9630941384425962</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B46" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C46" t="n">
-        <v>0.4508658786480607</v>
+        <v>0.4543573620020792</v>
       </c>
       <c r="D46" t="n">
-        <v>0.1124147219943875</v>
+        <v>0.1122061918405639</v>
       </c>
       <c r="E46" t="n">
-        <v>0.4367193993575518</v>
+        <v>0.4334364461573569</v>
       </c>
       <c r="F46" t="n">
         <v>1</v>
       </c>
       <c r="G46" t="n">
-        <v>0.01414647929050894</v>
+        <v>0.02092091584472222</v>
       </c>
       <c r="H46" t="n">
-        <v>0.9666487952468232</v>
+        <v>0.9662284464976205</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B47" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C47" t="n">
-        <v>0.4496424290138612</v>
+        <v>0.4531124014300565</v>
       </c>
       <c r="D47" t="n">
-        <v>0.114653141056062</v>
+        <v>0.1145896194122569</v>
       </c>
       <c r="E47" t="n">
-        <v>0.4357044299300769</v>
+        <v>0.4322979791576865</v>
       </c>
       <c r="F47" t="n">
         <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>0.01393799908378435</v>
+        <v>0.02081442227237001</v>
       </c>
       <c r="H47" t="n">
-        <v>0.9697005659212987</v>
+        <v>0.9694797731367073</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B48" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C48" t="n">
-        <v>0.4483174824369142</v>
+        <v>0.4518978675929917</v>
       </c>
       <c r="D48" t="n">
-        <v>0.1171329582518386</v>
+        <v>0.1168361266766399</v>
       </c>
       <c r="E48" t="n">
-        <v>0.4345495593112472</v>
+        <v>0.4312660057303684</v>
       </c>
       <c r="F48" t="n">
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>0.01376792312566694</v>
+        <v>0.02063186186262328</v>
       </c>
       <c r="H48" t="n">
-        <v>0.9730228607811582</v>
+        <v>0.9724949638986464</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B49" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C49" t="n">
-        <v>0.4470089948236559</v>
+        <v>0.4505869824285605</v>
       </c>
       <c r="D49" t="n">
-        <v>0.1197115292297479</v>
+        <v>0.1193209766981921</v>
       </c>
       <c r="E49" t="n">
-        <v>0.4332794759465962</v>
+        <v>0.4300920408732473</v>
       </c>
       <c r="F49" t="n">
         <v>1</v>
       </c>
       <c r="G49" t="n">
-        <v>0.01372951887705975</v>
+        <v>0.02049494155531323</v>
       </c>
       <c r="H49" t="n">
-        <v>0.9764122363774246</v>
+        <v>0.97577157896563</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B50" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C50" t="n">
-        <v>0.4455990102676502</v>
+        <v>0.4492887750703618</v>
       </c>
       <c r="D50" t="n">
-        <v>0.1223285044562644</v>
+        <v>0.1218869646796318</v>
       </c>
       <c r="E50" t="n">
-        <v>0.4320724852760854</v>
+        <v>0.4288242602500064</v>
       </c>
       <c r="F50" t="n">
         <v>1</v>
       </c>
       <c r="G50" t="n">
-        <v>0.01352652499156481</v>
+        <v>0.02046451482035544</v>
       </c>
       <c r="H50" t="n">
-        <v>0.9797901249660503</v>
+        <v>0.9790909395007259</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B51" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C51" t="n">
-        <v>0.4442521184057848</v>
+        <v>0.4478713963335784</v>
       </c>
       <c r="D51" t="n">
-        <v>0.1250058292163065</v>
+        <v>0.1245467684271914</v>
       </c>
       <c r="E51" t="n">
-        <v>0.4307420523779088</v>
+        <v>0.4275818352392302</v>
       </c>
       <c r="F51" t="n">
         <v>1</v>
       </c>
       <c r="G51" t="n">
-        <v>0.01351006602787597</v>
+        <v>0.02028956109434821</v>
       </c>
       <c r="H51" t="n">
-        <v>0.9831769406585473</v>
+        <v>0.982470072336568</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B52" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C52" t="n">
-        <v>0.4427982432799423</v>
+        <v>0.4465148710667106</v>
       </c>
       <c r="D52" t="n">
-        <v>0.1277819077584812</v>
+        <v>0.1272572833996805</v>
       </c>
       <c r="E52" t="n">
-        <v>0.4294198489615765</v>
+        <v>0.4262278455336089</v>
       </c>
       <c r="F52" t="n">
         <v>1</v>
       </c>
       <c r="G52" t="n">
-        <v>0.01337839431836574</v>
+        <v>0.02028702553310174</v>
       </c>
       <c r="H52" t="n">
-        <v>0.9866212510304491</v>
+        <v>0.9858427998499441</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B53" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C53" t="n">
-        <v>0.4411742921959824</v>
+        <v>0.4450898856461878</v>
       </c>
       <c r="D53" t="n">
-        <v>0.130799384434758</v>
+        <v>0.1300489363320571</v>
       </c>
       <c r="E53" t="n">
-        <v>0.4280263233692596</v>
+        <v>0.4248611780217551</v>
       </c>
       <c r="F53" t="n">
         <v>1</v>
       </c>
       <c r="G53" t="n">
-        <v>0.01314796882672276</v>
+        <v>0.02022870762443268</v>
       </c>
       <c r="H53" t="n">
-        <v>0.9902879908500148</v>
+        <v>0.9892486384657335</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B54" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C54" t="n">
-        <v>0.4396326359304664</v>
+        <v>0.4435026243058901</v>
       </c>
       <c r="D54" t="n">
-        <v>0.1337427957744354</v>
+        <v>0.1330383630416593</v>
       </c>
       <c r="E54" t="n">
-        <v>0.4266245682950983</v>
+        <v>0.4234590126524506</v>
       </c>
       <c r="F54" t="n">
         <v>1</v>
       </c>
       <c r="G54" t="n">
-        <v>0.0130080676353681</v>
+        <v>0.02004361165343949</v>
       </c>
       <c r="H54" t="n">
-        <v>0.9937862399760475</v>
+        <v>0.9928222572575354</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B55" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C55" t="n">
-        <v>0.4380388596132692</v>
+        <v>0.4419686097517685</v>
       </c>
       <c r="D55" t="n">
-        <v>0.1367630156113271</v>
+        <v>0.1359720074038388</v>
       </c>
       <c r="E55" t="n">
-        <v>0.4251981247754038</v>
+        <v>0.4220593828443926</v>
       </c>
       <c r="F55" t="n">
         <v>1</v>
       </c>
       <c r="G55" t="n">
-        <v>0.01284073483786546</v>
+        <v>0.01990922690737595</v>
       </c>
       <c r="H55" t="n">
-        <v>0.9972983938111872</v>
+        <v>0.9962527490305166</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B56" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C56" t="n">
-        <v>0.4363490726745542</v>
+        <v>0.4403737417277314</v>
       </c>
       <c r="D56" t="n">
-        <v>0.1399615408881806</v>
+        <v>0.1390121453383706</v>
       </c>
       <c r="E56" t="n">
-        <v>0.4236893864372653</v>
+        <v>0.4206141129338979</v>
       </c>
       <c r="F56" t="n">
         <v>1</v>
       </c>
       <c r="G56" t="n">
-        <v>0.01265968623728891</v>
+        <v>0.01975962879383347</v>
       </c>
       <c r="H56" t="n">
-        <v>1.000933716519817</v>
+        <v>0.9997307216310356</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B57" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C57" t="n">
-        <v>0.4346510562539947</v>
+        <v>0.4387078779887928</v>
       </c>
       <c r="D57" t="n">
-        <v>0.1432588199471667</v>
+        <v>0.1421892035802125</v>
       </c>
       <c r="E57" t="n">
-        <v>0.4220901237988385</v>
+        <v>0.4191029184309947</v>
       </c>
       <c r="F57" t="n">
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>0.01256093245515622</v>
+        <v>0.01960495955779812</v>
       </c>
       <c r="H57" t="n">
-        <v>1.004591016084537</v>
+        <v>1.003282787950767</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B58" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C58" t="n">
-        <v>0.4328734881756062</v>
+        <v>0.4370191941986359</v>
       </c>
       <c r="D58" t="n">
-        <v>0.1466932570368928</v>
+        <v>0.1454473997819417</v>
       </c>
       <c r="E58" t="n">
-        <v>0.420433254787501</v>
+        <v>0.4175334060194224</v>
       </c>
       <c r="F58" t="n">
         <v>1</v>
       </c>
       <c r="G58" t="n">
-        <v>0.01244023338810513</v>
+        <v>0.01948578817921348</v>
       </c>
       <c r="H58" t="n">
-        <v>1.008306539545091</v>
+        <v>1.006838718090966</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B59" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C59" t="n">
-        <v>0.4310931769366028</v>
+        <v>0.435246836887345</v>
       </c>
       <c r="D59" t="n">
-        <v>0.1501304372872336</v>
+        <v>0.1488526585359669</v>
       </c>
       <c r="E59" t="n">
-        <v>0.4187763857761636</v>
+        <v>0.415900504576688</v>
       </c>
       <c r="F59" t="n">
         <v>1</v>
       </c>
       <c r="G59" t="n">
-        <v>0.01231679116043921</v>
+        <v>0.01934633231065697</v>
       </c>
       <c r="H59" t="n">
-        <v>1.011930711912869</v>
+        <v>1.010464224664264</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B60" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C60" t="n">
-        <v>0.4292826909308367</v>
+        <v>0.4334541950860823</v>
       </c>
       <c r="D60" t="n">
-        <v>0.1537431798169215</v>
+        <v>0.1522959507086894</v>
       </c>
       <c r="E60" t="n">
-        <v>0.4169741292522419</v>
+        <v>0.4142498542052283</v>
       </c>
       <c r="F60" t="n">
         <v>1</v>
       </c>
       <c r="G60" t="n">
-        <v>0.01230856167859484</v>
+        <v>0.01920434088085399</v>
       </c>
       <c r="H60" t="n">
-        <v>1.015638446956844</v>
+        <v>1.01403717778734</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B61" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C61" t="n">
-        <v>0.4272801836820347</v>
+        <v>0.4316361976723548</v>
       </c>
       <c r="D61" t="n">
-        <v>0.157509539341038</v>
+        <v>0.1558812343112148</v>
       </c>
       <c r="E61" t="n">
-        <v>0.4152102769769273</v>
+        <v>0.4124825680164305</v>
       </c>
       <c r="F61" t="n">
         <v>1</v>
       </c>
       <c r="G61" t="n">
-        <v>0.01206990670510749</v>
+        <v>0.01915362965592432</v>
       </c>
       <c r="H61" t="n">
-        <v>1.01940037749027</v>
+        <v>1.017657687533946</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B62" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C62" t="n">
-        <v>0.4253188238424548</v>
+        <v>0.4296381754101271</v>
       </c>
       <c r="D62" t="n">
-        <v>0.1612868715076136</v>
+        <v>0.1596364005172545</v>
       </c>
       <c r="E62" t="n">
-        <v>0.4133943046499315</v>
+        <v>0.4107254240726185</v>
       </c>
       <c r="F62" t="n">
         <v>1</v>
       </c>
       <c r="G62" t="n">
-        <v>0.01192451919252324</v>
+        <v>0.01891275133750858</v>
       </c>
       <c r="H62" t="n">
-        <v>1.023064523536286</v>
+        <v>1.021349275172199</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B63" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C63" t="n">
-        <v>0.4232175628115202</v>
+        <v>0.4276604376378711</v>
       </c>
       <c r="D63" t="n">
-        <v>0.165352235538743</v>
+        <v>0.1634650979994422</v>
       </c>
       <c r="E63" t="n">
-        <v>0.4114302016497368</v>
+        <v>0.4088744643626867</v>
       </c>
       <c r="F63" t="n">
         <v>1</v>
       </c>
       <c r="G63" t="n">
-        <v>0.01178736116178336</v>
+        <v>0.01878597327518444</v>
       </c>
       <c r="H63" t="n">
-        <v>1.026889985701657</v>
+        <v>1.025002242522842</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B64" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C64" t="n">
-        <v>0.4211217881018152</v>
+        <v>0.4255280306295798</v>
       </c>
       <c r="D64" t="n">
-        <v>0.1695026375489311</v>
+        <v>0.1675752427799894</v>
       </c>
       <c r="E64" t="n">
-        <v>0.4093755743492537</v>
+        <v>0.4068967265904308</v>
       </c>
       <c r="F64" t="n">
         <v>1</v>
       </c>
       <c r="G64" t="n">
-        <v>0.01174621375256146</v>
+        <v>0.01863130403914903</v>
       </c>
       <c r="H64" t="n">
-        <v>1.030670536972532</v>
+        <v>1.028804888640144</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B65" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C65" t="n">
-        <v>0.4187681562943192</v>
+        <v>0.423403230305028</v>
       </c>
       <c r="D65" t="n">
-        <v>0.1739575303873617</v>
+        <v>0.1717234209792338</v>
       </c>
       <c r="E65" t="n">
-        <v>0.4072743133183191</v>
+        <v>0.4048733487157382</v>
       </c>
       <c r="F65" t="n">
         <v>1</v>
       </c>
       <c r="G65" t="n">
-        <v>0.01149384297600009</v>
+        <v>0.01852988158928981</v>
       </c>
       <c r="H65" t="n">
-        <v>1.034595258201808</v>
+        <v>1.032518702888822</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B66" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C66" t="n">
-        <v>0.4165242509114151</v>
+        <v>0.421019802733335</v>
       </c>
       <c r="D66" t="n">
-        <v>0.1784398548319403</v>
+        <v>0.1762164355079997</v>
       </c>
       <c r="E66" t="n">
-        <v>0.4050358942566446</v>
+        <v>0.4027637617586653</v>
       </c>
       <c r="F66" t="n">
         <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>0.01148835665477049</v>
+        <v>0.01825604097466971</v>
       </c>
       <c r="H66" t="n">
-        <v>1.038401268941652</v>
+        <v>1.036408473910636</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B67" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C67" t="n">
-        <v>0.4140800948036308</v>
+        <v>0.4187276553665154</v>
       </c>
       <c r="D67" t="n">
-        <v>0.1832431290684501</v>
+        <v>0.1807931235578995</v>
       </c>
       <c r="E67" t="n">
-        <v>0.4026767761279191</v>
+        <v>0.4004792210755851</v>
       </c>
       <c r="F67" t="n">
         <v>1</v>
       </c>
       <c r="G67" t="n">
-        <v>0.01140331867571176</v>
+        <v>0.01824843429093032</v>
       </c>
       <c r="H67" t="n">
-        <v>1.042328844982634</v>
+        <v>1.040221677508541</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B68" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C68" t="n">
-        <v>0.4114329448103516</v>
+        <v>0.4162554831511955</v>
       </c>
       <c r="D68" t="n">
-        <v>0.1882960309209064</v>
+        <v>0.1856182966099546</v>
       </c>
       <c r="E68" t="n">
-        <v>0.4002710242687419</v>
+        <v>0.3981262202388499</v>
       </c>
       <c r="F68" t="n">
         <v>1</v>
       </c>
       <c r="G68" t="n">
-        <v>0.01116192054160964</v>
+        <v>0.01812926291234568</v>
       </c>
       <c r="H68" t="n">
-        <v>1.046296304541695</v>
+        <v>1.044091273268426</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B69" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C69" t="n">
-        <v>0.4088461443505979</v>
+        <v>0.4136261061385938</v>
       </c>
       <c r="D69" t="n">
-        <v>0.1934833476434879</v>
+        <v>0.1906234945105099</v>
       </c>
       <c r="E69" t="n">
-        <v>0.3976705080059142</v>
+        <v>0.3957503993508963</v>
       </c>
       <c r="F69" t="n">
         <v>1</v>
       </c>
       <c r="G69" t="n">
-        <v>0.0111756363446836</v>
+        <v>0.01787570678769745</v>
       </c>
       <c r="H69" t="n">
-        <v>1.050191925647817</v>
+        <v>1.047945400449504</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B70" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C70" t="n">
-        <v>0.4060782952902676</v>
+        <v>0.4110322269834428</v>
       </c>
       <c r="D70" t="n">
-        <v>0.1988654287697199</v>
+        <v>0.1958061816983189</v>
       </c>
       <c r="E70" t="n">
-        <v>0.3950562759400126</v>
+        <v>0.3931615913182383</v>
       </c>
       <c r="F70" t="n">
         <v>1</v>
       </c>
       <c r="G70" t="n">
-        <v>0.01102201935025499</v>
+        <v>0.01787063566520447</v>
       </c>
       <c r="H70" t="n">
-        <v>1.054053888820583</v>
+        <v>1.051759402153754</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B71" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C71" t="n">
-        <v>0.4032775283025596</v>
+        <v>0.4082583229797916</v>
       </c>
       <c r="D71" t="n">
-        <v>0.2043215752325514</v>
+        <v>0.2011790359796141</v>
       </c>
       <c r="E71" t="n">
-        <v>0.3924008964648889</v>
+        <v>0.3905626410405943</v>
       </c>
       <c r="F71" t="n">
         <v>1</v>
       </c>
       <c r="G71" t="n">
-        <v>0.01087663183767074</v>
+        <v>0.01769568193919724</v>
       </c>
       <c r="H71" t="n">
-        <v>1.05778325966735</v>
+        <v>1.055537057068804</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B72" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C72" t="n">
-        <v>0.4003286306416527</v>
+        <v>0.4054742767311544</v>
       </c>
       <c r="D72" t="n">
-        <v>0.2101096441297735</v>
+        <v>0.2065772458733741</v>
       </c>
       <c r="E72" t="n">
-        <v>0.3895617252285739</v>
+        <v>0.3879484773954715</v>
       </c>
       <c r="F72" t="n">
         <v>1</v>
       </c>
       <c r="G72" t="n">
-        <v>0.01076690541307884</v>
+        <v>0.01752579933568293</v>
       </c>
       <c r="H72" t="n">
-        <v>1.061538791303916</v>
+        <v>1.059151490286558</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B73" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C73" t="n">
-        <v>0.3973824761413606</v>
+        <v>0.4025304901239889</v>
       </c>
       <c r="D73" t="n">
-        <v>0.2159772646848246</v>
+        <v>0.2123355054641345</v>
       </c>
       <c r="E73" t="n">
-        <v>0.3866402591738149</v>
+        <v>0.3851340044118766</v>
       </c>
       <c r="F73" t="n">
         <v>1</v>
       </c>
       <c r="G73" t="n">
-        <v>0.01074221696754568</v>
+        <v>0.01739648571211239</v>
       </c>
       <c r="H73" t="n">
-        <v>1.065138712066902</v>
+        <v>1.062809940447977</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B74" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C74" t="n">
-        <v>0.3943430541801653</v>
+        <v>0.3995841679555769</v>
       </c>
       <c r="D74" t="n">
-        <v>0.2217927651881945</v>
+        <v>0.2182535054134233</v>
       </c>
       <c r="E74" t="n">
-        <v>0.3838641806316402</v>
+        <v>0.3821623266309997</v>
       </c>
       <c r="F74" t="n">
         <v>1</v>
       </c>
       <c r="G74" t="n">
-        <v>0.01047887354852511</v>
+        <v>0.01742184132457719</v>
       </c>
       <c r="H74" t="n">
-        <v>1.068509251848376</v>
+        <v>1.066359807126148</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B75" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C75" t="n">
-        <v>0.3911884194731486</v>
+        <v>0.3965389588985522</v>
       </c>
       <c r="D75" t="n">
-        <v>0.2280142534625545</v>
+        <v>0.2240878318415781</v>
       </c>
       <c r="E75" t="n">
-        <v>0.3807973270642969</v>
+        <v>0.3793732092598697</v>
       </c>
       <c r="F75" t="n">
         <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>0.01039109240885167</v>
+        <v>0.0171657496386825</v>
       </c>
       <c r="H75" t="n">
-        <v>1.07189559183761</v>
+        <v>1.069664748729356</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B76" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C76" t="n">
-        <v>0.3879734352326063</v>
+        <v>0.3934100763203935</v>
       </c>
       <c r="D76" t="n">
-        <v>0.2343701566070395</v>
+        <v>0.2302669945992545</v>
       </c>
       <c r="E76" t="n">
-        <v>0.3776564081603542</v>
+        <v>0.3763229290803519</v>
       </c>
       <c r="F76" t="n">
         <v>1</v>
       </c>
       <c r="G76" t="n">
-        <v>0.01031702707225213</v>
+        <v>0.01708714724004162</v>
       </c>
       <c r="H76" t="n">
-        <v>1.07512781832167</v>
+        <v>1.072947339693878</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B77" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C77" t="n">
-        <v>0.3845033370548879</v>
+        <v>0.3901594868024037</v>
       </c>
       <c r="D77" t="n">
-        <v>0.241030550579767</v>
+        <v>0.2366135043991988</v>
       </c>
       <c r="E77" t="n">
-        <v>0.3744661123653451</v>
+        <v>0.3732270087983975</v>
       </c>
       <c r="F77" t="n">
         <v>1</v>
       </c>
       <c r="G77" t="n">
-        <v>0.01003722468954282</v>
+        <v>0.01693247800400616</v>
       </c>
       <c r="H77" t="n">
-        <v>1.078276073070528</v>
+        <v>1.076096235881801</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B78" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C78" t="n">
-        <v>0.3810030641104067</v>
+        <v>0.3866933745784629</v>
       </c>
       <c r="D78" t="n">
-        <v>0.2480310964687293</v>
+        <v>0.2432287836912701</v>
       </c>
       <c r="E78" t="n">
-        <v>0.3709658394208639</v>
+        <v>0.370077841730267</v>
       </c>
       <c r="F78" t="n">
         <v>1</v>
       </c>
       <c r="G78" t="n">
-        <v>0.01003722468954282</v>
+        <v>0.01661553284819595</v>
       </c>
       <c r="H78" t="n">
-        <v>1.08131985957876</v>
+        <v>1.079144603908279</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B79" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C79" t="n">
-        <v>0.3772778519955122</v>
+        <v>0.3831740155683461</v>
       </c>
       <c r="D79" t="n">
-        <v>0.2552318930825719</v>
+        <v>0.2502091838028347</v>
       </c>
       <c r="E79" t="n">
-        <v>0.3674902549219159</v>
+        <v>0.3666168006288192</v>
       </c>
       <c r="F79" t="n">
         <v>1</v>
       </c>
       <c r="G79" t="n">
-        <v>0.009787597073596221</v>
+        <v>0.01655721493952689</v>
       </c>
       <c r="H79" t="n">
-        <v>1.084179903424149</v>
+        <v>1.082097400346168</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B80" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C80" t="n">
-        <v>0.373453886098485</v>
+        <v>0.3794492760972641</v>
       </c>
       <c r="D80" t="n">
-        <v>0.2626192246182206</v>
+        <v>0.2573848221303786</v>
       </c>
       <c r="E80" t="n">
-        <v>0.3639268892832944</v>
+        <v>0.3631659017723573</v>
       </c>
       <c r="F80" t="n">
         <v>1</v>
       </c>
       <c r="G80" t="n">
-        <v>0.009526996815190536</v>
+        <v>0.01628337432490684</v>
       </c>
       <c r="H80" t="n">
-        <v>1.08683061010501</v>
+        <v>1.084866787291237</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B81" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C81" t="n">
-        <v>0.3694488716008811</v>
+        <v>0.3756611475950202</v>
       </c>
       <c r="D81" t="n">
-        <v>0.2703439649094894</v>
+        <v>0.2647328786226831</v>
       </c>
       <c r="E81" t="n">
-        <v>0.3602071634896295</v>
+        <v>0.3596059737822967</v>
       </c>
       <c r="F81" t="n">
         <v>1</v>
       </c>
       <c r="G81" t="n">
-        <v>0.009241708111251579</v>
+        <v>0.01605517381272348</v>
       </c>
       <c r="H81" t="n">
-        <v>1.089301147270179</v>
+        <v>1.087422399704189</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B82" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C82" t="n">
-        <v>0.3654219118183589</v>
+        <v>0.371624534090621</v>
       </c>
       <c r="D82" t="n">
-        <v>0.2781372842161282</v>
+        <v>0.2724435203732346</v>
       </c>
       <c r="E82" t="n">
-        <v>0.356440803965513</v>
+        <v>0.3559319455361444</v>
       </c>
       <c r="F82" t="n">
         <v>1</v>
       </c>
       <c r="G82" t="n">
-        <v>0.008981107852845893</v>
+        <v>0.01569258855447653</v>
       </c>
       <c r="H82" t="n">
-        <v>1.091486668959312</v>
+        <v>1.089808573222043</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B83" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C83" t="n">
-        <v>0.3611782423472677</v>
+        <v>0.3675777783412358</v>
       </c>
       <c r="D83" t="n">
-        <v>0.2863667660605196</v>
+        <v>0.2802784046248637</v>
       </c>
       <c r="E83" t="n">
-        <v>0.3524549915922127</v>
+        <v>0.3521438170339005</v>
       </c>
       <c r="F83" t="n">
         <v>1</v>
       </c>
       <c r="G83" t="n">
-        <v>0.008723250755054979</v>
+        <v>0.01543396130733538</v>
       </c>
       <c r="H83" t="n">
-        <v>1.093465952171546</v>
+        <v>1.091923561039145</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B84" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C84" t="n">
-        <v>0.3569455455186357</v>
+        <v>0.3633028220796674</v>
       </c>
       <c r="D84" t="n">
-        <v>0.2945660731381483</v>
+        <v>0.2885291209209159</v>
       </c>
       <c r="E84" t="n">
-        <v>0.348488381343216</v>
+        <v>0.3481680569994168</v>
       </c>
       <c r="F84" t="n">
         <v>1</v>
       </c>
       <c r="G84" t="n">
-        <v>0.00845716417541964</v>
+        <v>0.01513476508025052</v>
       </c>
       <c r="H84" t="n">
-        <v>1.09510843673517</v>
+        <v>1.093822463517941</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B85" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C85" t="n">
-        <v>0.3524851663589755</v>
+        <v>0.3590278658180988</v>
       </c>
       <c r="D85" t="n">
-        <v>0.3032070290747594</v>
+        <v>0.2967494104820102</v>
       </c>
       <c r="E85" t="n">
-        <v>0.3443078045662651</v>
+        <v>0.344222723699891</v>
       </c>
       <c r="F85" t="n">
         <v>1</v>
       </c>
       <c r="G85" t="n">
-        <v>0.008177361792710336</v>
+        <v>0.01480514211820783</v>
       </c>
       <c r="H85" t="n">
-        <v>1.096489267808185</v>
+        <v>1.095385180922227</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B86" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C86" t="n">
-        <v>0.3479726671476341</v>
+        <v>0.354588098075509</v>
       </c>
       <c r="D86" t="n">
-        <v>0.3122704317460492</v>
+        <v>0.3053398919850909</v>
       </c>
       <c r="E86" t="n">
-        <v>0.3397569011063167</v>
+        <v>0.3400720099394001</v>
       </c>
       <c r="F86" t="n">
         <v>1</v>
       </c>
       <c r="G86" t="n">
-        <v>0.008215766041317463</v>
+        <v>0.01451608813610894</v>
       </c>
       <c r="H86" t="n">
-        <v>1.097553980505716</v>
+        <v>1.096671129340864</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B87" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C87" t="n">
-        <v>0.343078868610836</v>
+        <v>0.3500469078830599</v>
       </c>
       <c r="D87" t="n">
-        <v>0.3217727401157065</v>
+        <v>0.31436395446132</v>
       </c>
       <c r="E87" t="n">
-        <v>0.3351483912734575</v>
+        <v>0.3355891376556201</v>
       </c>
       <c r="F87" t="n">
         <v>1</v>
       </c>
       <c r="G87" t="n">
-        <v>0.007930477337378561</v>
+        <v>0.01445777022743983</v>
       </c>
       <c r="H87" t="n">
-        <v>1.098263428625466</v>
+        <v>1.097642190753805</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B88" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C88" t="n">
-        <v>0.3381274637011272</v>
+        <v>0.3451811658510611</v>
       </c>
       <c r="D88" t="n">
-        <v>0.3314670697283997</v>
+        <v>0.3237734222470144</v>
       </c>
       <c r="E88" t="n">
-        <v>0.3304054665704731</v>
+        <v>0.3310454119019245</v>
       </c>
       <c r="F88" t="n">
         <v>1</v>
       </c>
       <c r="G88" t="n">
-        <v>0.007721997130654024</v>
+        <v>0.01413575394913663</v>
       </c>
       <c r="H88" t="n">
-        <v>1.098559843633459</v>
+        <v>1.098257892771608</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B89" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C89" t="n">
-        <v>0.3329785512271529</v>
+        <v>0.340224143614189</v>
       </c>
       <c r="D89" t="n">
-        <v>0.3415619007908532</v>
+        <v>0.3334491239635893</v>
       </c>
       <c r="E89" t="n">
-        <v>0.3254595479819939</v>
+        <v>0.3263267324222217</v>
       </c>
       <c r="F89" t="n">
         <v>1</v>
       </c>
       <c r="G89" t="n">
-        <v>0.007519003245159028</v>
+        <v>0.01389741119196736</v>
       </c>
       <c r="H89" t="n">
-        <v>1.09841762263629</v>
+        <v>1.09846736631271</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B90" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C90" t="n">
-        <v>0.3274154215003443</v>
+        <v>0.3350845609675702</v>
       </c>
       <c r="D90" t="n">
-        <v>0.3522355387430289</v>
+        <v>0.3435685488982986</v>
       </c>
       <c r="E90" t="n">
-        <v>0.3203490397566268</v>
+        <v>0.3213468901341312</v>
       </c>
       <c r="F90" t="n">
         <v>1</v>
       </c>
       <c r="G90" t="n">
-        <v>0.007066381743717487</v>
+        <v>0.01373767083343896</v>
       </c>
       <c r="H90" t="n">
-        <v>1.097777115179991</v>
+        <v>1.098233995230155</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B91" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C91" t="n">
-        <v>0.3219949361255051</v>
+        <v>0.3294860417353381</v>
       </c>
       <c r="D91" t="n">
-        <v>0.362958553586271</v>
+        <v>0.3542610106747128</v>
       </c>
       <c r="E91" t="n">
-        <v>0.3150465102882239</v>
+        <v>0.316252947589949</v>
       </c>
       <c r="F91" t="n">
         <v>1</v>
       </c>
       <c r="G91" t="n">
-        <v>0.006948425837281169</v>
+        <v>0.01323309414538909</v>
       </c>
       <c r="H91" t="n">
-        <v>1.096627052060483</v>
+        <v>1.097501096744616</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B92" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C92" t="n">
-        <v>0.3160395344307805</v>
+        <v>0.3239864093917189</v>
       </c>
       <c r="D92" t="n">
-        <v>0.3742411731949317</v>
+        <v>0.3650168614822891</v>
       </c>
       <c r="E92" t="n">
-        <v>0.3097192923742878</v>
+        <v>0.310996729125992</v>
       </c>
       <c r="F92" t="n">
         <v>1</v>
       </c>
       <c r="G92" t="n">
-        <v>0.006320242056492675</v>
+        <v>0.01298968026572683</v>
       </c>
       <c r="H92" t="n">
-        <v>1.094885426589823</v>
+        <v>1.096254103373779</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B93" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C93" t="n">
-        <v>0.3099497178659308</v>
+        <v>0.3179898070437892</v>
       </c>
       <c r="D93" t="n">
-        <v>0.3862095829572917</v>
+        <v>0.3762823601004082</v>
       </c>
       <c r="E93" t="n">
-        <v>0.3038406991767775</v>
+        <v>0.3057278328558026</v>
       </c>
       <c r="F93" t="n">
         <v>1</v>
       </c>
       <c r="G93" t="n">
-        <v>0.006109018689153312</v>
+        <v>0.01226197418798652</v>
       </c>
       <c r="H93" t="n">
-        <v>1.092439047519332</v>
+        <v>1.094422374678815</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B94" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C94" t="n">
-        <v>0.3036404484518973</v>
+        <v>0.3118816400010142</v>
       </c>
       <c r="D94" t="n">
-        <v>0.3983782434445319</v>
+        <v>0.3882045690813661</v>
       </c>
       <c r="E94" t="n">
-        <v>0.2979813081035708</v>
+        <v>0.2999137909176196</v>
       </c>
       <c r="F94" t="n">
         <v>1</v>
       </c>
       <c r="G94" t="n">
-        <v>0.005659140348326541</v>
+        <v>0.0119678490833946</v>
       </c>
       <c r="H94" t="n">
-        <v>1.089334424113648</v>
+        <v>1.091885400773082</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B95" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C95" t="n">
-        <v>0.2969553660336366</v>
+        <v>0.3055579502522883</v>
       </c>
       <c r="D95" t="n">
-        <v>0.4113369341888337</v>
+        <v>0.4003854053094653</v>
       </c>
       <c r="E95" t="n">
-        <v>0.2917076997775297</v>
+        <v>0.2940566444382464</v>
       </c>
       <c r="F95" t="n">
         <v>1</v>
       </c>
       <c r="G95" t="n">
-        <v>0.005247666256106953</v>
+        <v>0.01150130581404191</v>
       </c>
       <c r="H95" t="n">
-        <v>1.085348201989514</v>
+        <v>1.088678477746841</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B96" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C96" t="n">
-        <v>0.2899465906628299</v>
+        <v>0.2988767463678085</v>
       </c>
       <c r="D96" t="n">
-        <v>0.4246412631705999</v>
+        <v>0.4132559141966074</v>
       </c>
       <c r="E96" t="n">
-        <v>0.2854121461665702</v>
+        <v>0.2878673394355841</v>
       </c>
       <c r="F96" t="n">
         <v>1</v>
       </c>
       <c r="G96" t="n">
-        <v>0.004534444496259726</v>
+        <v>0.01100940693222446</v>
       </c>
       <c r="H96" t="n">
-        <v>1.080536321034866</v>
+        <v>1.084618404286455</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B97" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C97" t="n">
-        <v>0.2829405584526379</v>
+        <v>0.2918735262050255</v>
       </c>
       <c r="D97" t="n">
-        <v>0.4385490874876215</v>
+        <v>0.4265397195669262</v>
       </c>
       <c r="E97" t="n">
-        <v>0.2785103540597406</v>
+        <v>0.2815867542280484</v>
       </c>
       <c r="F97" t="n">
         <v>1</v>
       </c>
       <c r="G97" t="n">
-        <v>0.004430204392897374</v>
+        <v>0.01028677197697714</v>
       </c>
       <c r="H97" t="n">
-        <v>1.07472625767152</v>
+        <v>1.079715293578948</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B98" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C98" t="n">
-        <v>0.275555970077604</v>
+        <v>0.2847714191536296</v>
       </c>
       <c r="D98" t="n">
-        <v>0.4528409542907147</v>
+        <v>0.4404371307588935</v>
       </c>
       <c r="E98" t="n">
-        <v>0.2716030756316813</v>
+        <v>0.2747914500874769</v>
       </c>
       <c r="F98" t="n">
         <v>1</v>
       </c>
       <c r="G98" t="n">
-        <v>0.003952894445922728</v>
+        <v>0.009979969066152783</v>
       </c>
       <c r="H98" t="n">
-        <v>1.067940079126627</v>
+        <v>1.07380525147594</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B99" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C99" t="n">
-        <v>0.2680451963142894</v>
+        <v>0.2773143335277264</v>
       </c>
       <c r="D99" t="n">
-        <v>0.4678487860142699</v>
+        <v>0.4547478384340374</v>
       </c>
       <c r="E99" t="n">
-        <v>0.2641060176714407</v>
+        <v>0.2679378280382362</v>
       </c>
       <c r="F99" t="n">
         <v>1</v>
       </c>
       <c r="G99" t="n">
-        <v>0.003939178642848706</v>
+        <v>0.00937650548949015</v>
       </c>
       <c r="H99" t="n">
-        <v>1.059922883210434</v>
+        <v>1.066905424134982</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B100" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C100" t="n">
-        <v>0.2599720746249414</v>
+        <v>0.2697355409619919</v>
       </c>
       <c r="D100" t="n">
-        <v>0.4834875446792285</v>
+        <v>0.4696899008595553</v>
       </c>
       <c r="E100" t="n">
-        <v>0.2565403806958301</v>
+        <v>0.2605745581784528</v>
       </c>
       <c r="F100" t="n">
         <v>1</v>
       </c>
       <c r="G100" t="n">
-        <v>0.003431693929111246</v>
+        <v>0.009160982783539107</v>
       </c>
       <c r="H100" t="n">
-        <v>1.05060950803757</v>
+        <v>1.058812465520779</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B101" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C101" t="n">
-        <v>0.2517892265110014</v>
+        <v>0.2615684981870737</v>
       </c>
       <c r="D101" t="n">
-        <v>0.4995706953637842</v>
+        <v>0.4853317781891022</v>
       </c>
       <c r="E101" t="n">
-        <v>0.2486400781252143</v>
+        <v>0.2530997236238242</v>
       </c>
       <c r="F101" t="n">
         <v>1</v>
       </c>
       <c r="G101" t="n">
-        <v>0.003149148385787143</v>
+        <v>0.00846877456324957</v>
       </c>
       <c r="H101" t="n">
-        <v>1.040008061839811</v>
+        <v>1.049387949986889</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B102" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C102" t="n">
-        <v>0.2432168495897603</v>
+        <v>0.2533862420446766</v>
       </c>
       <c r="D102" t="n">
-        <v>0.5161037243891667</v>
+        <v>0.5013108851644311</v>
       </c>
       <c r="E102" t="n">
-        <v>0.240679426021073</v>
+        <v>0.2453028727908923</v>
       </c>
       <c r="F102" t="n">
         <v>1</v>
       </c>
       <c r="G102" t="n">
-        <v>0.002537423568687386</v>
+        <v>0.008083369253784306</v>
       </c>
       <c r="H102" t="n">
-        <v>1.02803311427989</v>
+        <v>1.038743179153767</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B103" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C103" t="n">
-        <v>0.2345621778500753</v>
+        <v>0.2448388650827861</v>
       </c>
       <c r="D103" t="n">
-        <v>0.5330399980249244</v>
+        <v>0.5177844265828241</v>
       </c>
       <c r="E103" t="n">
-        <v>0.2323978241250003</v>
+        <v>0.2373767083343898</v>
       </c>
       <c r="F103" t="n">
         <v>1</v>
       </c>
       <c r="G103" t="n">
-        <v>0.002164353725074952</v>
+        <v>0.007462156748396259</v>
       </c>
       <c r="H103" t="n">
-        <v>1.014629295840312</v>
+        <v>1.026703097846176</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B104" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C104" t="n">
-        <v>0.2255316931061631</v>
+        <v>0.2360404675574939</v>
       </c>
       <c r="D104" t="n">
-        <v>0.5508239082906543</v>
+        <v>0.5347802936179924</v>
       </c>
       <c r="E104" t="n">
-        <v>0.2236443986031826</v>
+        <v>0.2291792388245138</v>
       </c>
       <c r="F104" t="n">
         <v>1</v>
       </c>
       <c r="G104" t="n">
-        <v>0.001887294502980447</v>
+        <v>0.006861228732980063</v>
       </c>
       <c r="H104" t="n">
-        <v>0.9993132815748889</v>
+        <v>1.013141015102688</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B105" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C105" t="n">
-        <v>0.2160540731820389</v>
+        <v>0.2268820203352012</v>
       </c>
       <c r="D105" t="n">
-        <v>0.5692387454977876</v>
+        <v>0.5525951469357743</v>
       </c>
       <c r="E105" t="n">
-        <v>0.2147071813201735</v>
+        <v>0.2205228327290246</v>
       </c>
       <c r="F105" t="n">
         <v>1</v>
       </c>
       <c r="G105" t="n">
-        <v>0.001346891861865401</v>
+        <v>0.006359187606176625</v>
       </c>
       <c r="H105" t="n">
-        <v>0.9821071323537554</v>
+        <v>0.9976766481229895</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B106" t="n">
+        <v>22</v>
+      </c>
+      <c r="C106" t="n">
+        <v>0.2173407033646898</v>
+      </c>
+      <c r="D106" t="n">
+        <v>0.5710058571464793</v>
+      </c>
+      <c r="E106" t="n">
+        <v>0.2116534394888309</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0.005687263875858911</v>
+      </c>
+      <c r="H106" t="n">
+        <v>0.9803477251070029</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="B106" t="n">
+      <c r="B107" t="n">
         <v>21</v>
       </c>
-      <c r="C106" t="n">
-        <v>0.2061238317564732</v>
-      </c>
-      <c r="D106" t="n">
-        <v>0.5883064549312427</v>
-      </c>
-      <c r="E106" t="n">
-        <v>0.2055697133122842</v>
-      </c>
-      <c r="F106" t="n">
-        <v>1</v>
-      </c>
-      <c r="G106" t="n">
-        <v>0.0005541184441890112</v>
-      </c>
-      <c r="H106" t="n">
-        <v>0.9628328568275604</v>
+      <c r="C107" t="n">
+        <v>0.2072745252161566</v>
+      </c>
+      <c r="D107" t="n">
+        <v>0.5901442734349248</v>
+      </c>
+      <c r="E107" t="n">
+        <v>0.2025812013489186</v>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0.004693323867238031</v>
+      </c>
+      <c r="H107" t="n">
+        <v>0.9608694588888901</v>
       </c>
     </row>
   </sheetData>

</xml_diff>